<commit_message>
revoke the Commit aeab14c by removing sample_id from component file
</commit_message>
<xml_diff>
--- a/single_cell/singlecell_schema_main_v0.4.xlsx
+++ b/single_cell/singlecell_schema_main_v0.4.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/providen/Documents/EI/Projects/COPO-schemas/single_cell/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zef22hak/development/COPO-schemas/single_cell/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51FE860A-E306-A64B-A85A-EAD734F8A124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A716B4C-E7AD-5149-A9F8-6706772BBE40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35800" yWindow="60" windowWidth="30240" windowHeight="17960" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
     <sheet name="term_mapping" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">data!$A$1:$S$202</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">data!$A$1:$S$201</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">regex_to_formula!$A$1:$C$53</definedName>
     <definedName name="Z_D34CFE6F_6B19_C846_A6A5_7A3E0DEDB173_.wvu.FilterData" localSheetId="0" hidden="1">data!$A$1:$S$163</definedName>
   </definedNames>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3136" uniqueCount="1267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3123" uniqueCount="1267">
   <si>
     <t>component_name</t>
   </si>
@@ -5028,7 +5028,7 @@
 <file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
 <namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <namedSheetView name="View1" id="{6954CA39-3A4A-425E-8D74-F55DAFA5B207}">
-    <nsvFilter filterId="{545CA0C1-0282-3A43-9C60-512DE414A571}" ref="A1:S202" tableId="0"/>
+    <nsvFilter filterId="{545CA0C1-0282-3A43-9C60-512DE414A571}" ref="A1:S201" tableId="0"/>
   </namedSheetView>
 </namedSheetViews>
 </file>
@@ -5378,7 +5378,7 @@
   <sheetPr>
     <tabColor theme="5" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:S203"/>
+  <dimension ref="A1:S202"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
@@ -12912,7 +12912,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="166" spans="1:19" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" s="8" t="s">
         <v>519</v>
       </c>
@@ -12920,25 +12920,29 @@
         <v>19</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>150</v>
+        <v>278</v>
       </c>
       <c r="D166" s="3" t="s">
-        <v>151</v>
+        <v>279</v>
       </c>
       <c r="F166" s="1" t="b">
         <v>0</v>
       </c>
       <c r="H166" s="1" t="s">
-        <v>148</v>
+        <v>277</v>
       </c>
       <c r="I166" s="3" t="s">
-        <v>1264</v>
+        <v>280</v>
       </c>
       <c r="J166" s="3" t="s">
-        <v>1251</v>
-      </c>
-      <c r="K166" s="3"/>
-      <c r="L166" s="3"/>
+        <v>1252</v>
+      </c>
+      <c r="K166" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="L166" s="3" t="s">
+        <v>1224</v>
+      </c>
       <c r="M166" s="3" t="s">
         <v>24</v>
       </c>
@@ -12967,22 +12971,22 @@
         <v>19</v>
       </c>
       <c r="C167" s="3" t="s">
-        <v>278</v>
+        <v>436</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>279</v>
+        <v>437</v>
       </c>
       <c r="F167" s="1" t="b">
         <v>0</v>
       </c>
       <c r="H167" s="1" t="s">
-        <v>277</v>
+        <v>435</v>
       </c>
       <c r="I167" s="3" t="s">
-        <v>280</v>
+        <v>438</v>
       </c>
       <c r="J167" s="3" t="s">
-        <v>1252</v>
+        <v>1253</v>
       </c>
       <c r="K167" s="3" t="s">
         <v>23</v>
@@ -13018,34 +13022,27 @@
         <v>19</v>
       </c>
       <c r="C168" s="3" t="s">
-        <v>436</v>
+        <v>684</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>437</v>
+        <v>685</v>
       </c>
       <c r="F168" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H168" s="1" t="s">
-        <v>435</v>
-      </c>
       <c r="I168" s="3" t="s">
-        <v>438</v>
+        <v>686</v>
       </c>
       <c r="J168" s="3" t="s">
-        <v>1253</v>
-      </c>
-      <c r="K168" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="L168" s="3" t="s">
-        <v>1224</v>
-      </c>
+        <v>687</v>
+      </c>
+      <c r="K168" s="3"/>
+      <c r="L168" s="3"/>
       <c r="M168" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N168" s="3" t="s">
-        <v>25</v>
+        <v>519</v>
       </c>
       <c r="O168" s="3"/>
       <c r="P168" s="31" t="s">
@@ -13069,19 +13066,19 @@
         <v>19</v>
       </c>
       <c r="C169" s="3" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="F169" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I169" s="3" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="J169" s="3" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="K169" s="3"/>
       <c r="L169" s="3"/>
@@ -13093,16 +13090,16 @@
       </c>
       <c r="O169" s="3"/>
       <c r="P169" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q169" s="56" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R169" s="56" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S169" s="85" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="170" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -13113,19 +13110,19 @@
         <v>19</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="F170" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I170" s="3" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="J170" s="3" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="K170" s="3"/>
       <c r="L170" s="3"/>
@@ -13133,7 +13130,7 @@
         <v>24</v>
       </c>
       <c r="N170" s="3" t="s">
-        <v>519</v>
+        <v>25</v>
       </c>
       <c r="O170" s="3"/>
       <c r="P170" s="31" t="s">
@@ -13157,19 +13154,19 @@
         <v>19</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="F171" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I171" s="3" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="J171" s="3" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="K171" s="3"/>
       <c r="L171" s="3"/>
@@ -13183,13 +13180,13 @@
       <c r="P171" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="Q171" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="R171" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="S171" s="85" t="s">
+      <c r="Q171" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="R171" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="S171" s="31" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13201,22 +13198,26 @@
         <v>19</v>
       </c>
       <c r="C172" s="3" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="D172" s="3" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="F172" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I172" s="3" t="s">
-        <v>698</v>
-      </c>
-      <c r="J172" s="3" t="s">
-        <v>699</v>
-      </c>
-      <c r="K172" s="3"/>
-      <c r="L172" s="3"/>
+        <v>702</v>
+      </c>
+      <c r="J172" s="41" t="s">
+        <v>1242</v>
+      </c>
+      <c r="K172" s="3" t="s">
+        <v>1213</v>
+      </c>
+      <c r="L172" s="3" t="s">
+        <v>1237</v>
+      </c>
       <c r="M172" s="3" t="s">
         <v>24</v>
       </c>
@@ -13225,16 +13226,16 @@
       </c>
       <c r="O172" s="3"/>
       <c r="P172" s="31" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q172" s="31" t="s">
-        <v>27</v>
-      </c>
-      <c r="R172" s="31" t="s">
-        <v>27</v>
-      </c>
-      <c r="S172" s="31" t="s">
-        <v>27</v>
+        <v>26</v>
+      </c>
+      <c r="Q172" s="56" t="s">
+        <v>26</v>
+      </c>
+      <c r="R172" s="56" t="s">
+        <v>26</v>
+      </c>
+      <c r="S172" s="85" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="173" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -13245,19 +13246,19 @@
         <v>19</v>
       </c>
       <c r="C173" s="3" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
       <c r="D173" s="3" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
       <c r="F173" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I173" s="3" t="s">
-        <v>702</v>
-      </c>
-      <c r="J173" s="41" t="s">
-        <v>1242</v>
+        <v>705</v>
+      </c>
+      <c r="J173" s="93" t="s">
+        <v>1241</v>
       </c>
       <c r="K173" s="3" t="s">
         <v>1213</v>
@@ -13273,19 +13274,19 @@
       </c>
       <c r="O173" s="3"/>
       <c r="P173" s="31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q173" s="56" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R173" s="56" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S173" s="85" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="174" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="174" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A174" s="8" t="s">
         <v>519</v>
       </c>
@@ -13293,31 +13294,27 @@
         <v>19</v>
       </c>
       <c r="C174" s="3" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
       <c r="D174" s="3" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="F174" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I174" s="3" t="s">
-        <v>705</v>
-      </c>
-      <c r="J174" s="93" t="s">
-        <v>1241</v>
-      </c>
-      <c r="K174" s="3" t="s">
-        <v>1213</v>
-      </c>
-      <c r="L174" s="3" t="s">
-        <v>1237</v>
-      </c>
+        <v>708</v>
+      </c>
+      <c r="J174" s="3" t="s">
+        <v>709</v>
+      </c>
+      <c r="K174" s="3"/>
+      <c r="L174" s="3"/>
       <c r="M174" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N174" s="3" t="s">
-        <v>25</v>
+        <v>519</v>
       </c>
       <c r="O174" s="3"/>
       <c r="P174" s="31" t="s">
@@ -13333,104 +13330,110 @@
         <v>27</v>
       </c>
     </row>
-    <row r="175" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A175" s="8" t="s">
-        <v>519</v>
-      </c>
-      <c r="B175" s="3" t="s">
+    <row r="175" spans="1:19" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A175" s="45" t="s">
+        <v>1108</v>
+      </c>
+      <c r="B175" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="C175" s="3" t="s">
-        <v>706</v>
-      </c>
-      <c r="D175" s="3" t="s">
-        <v>707</v>
-      </c>
-      <c r="F175" s="1" t="b">
+      <c r="C175" s="44" t="s">
+        <v>20</v>
+      </c>
+      <c r="D175" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="E175" s="44"/>
+      <c r="F175" s="46" t="b">
         <v>0</v>
       </c>
-      <c r="I175" s="3" t="s">
-        <v>708</v>
-      </c>
-      <c r="J175" s="3" t="s">
-        <v>709</v>
-      </c>
-      <c r="K175" s="3"/>
-      <c r="L175" s="3"/>
-      <c r="M175" s="3" t="s">
+      <c r="G175" s="46"/>
+      <c r="H175" s="46" t="s">
+        <v>18</v>
+      </c>
+      <c r="I175" s="44" t="s">
+        <v>22</v>
+      </c>
+      <c r="J175" s="44" t="s">
+        <v>1249</v>
+      </c>
+      <c r="K175" s="44" t="s">
+        <v>23</v>
+      </c>
+      <c r="L175" s="44" t="s">
+        <v>1224</v>
+      </c>
+      <c r="M175" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="N175" s="3" t="s">
-        <v>519</v>
-      </c>
-      <c r="O175" s="3"/>
-      <c r="P175" s="31" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q175" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="R175" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="S175" s="85" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="176" spans="1:19" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A176" s="45" t="s">
+      <c r="N175" s="44" t="s">
+        <v>25</v>
+      </c>
+      <c r="O175" s="44"/>
+      <c r="P175" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q175" s="62" t="s">
+        <v>26</v>
+      </c>
+      <c r="R175" s="62" t="s">
+        <v>26</v>
+      </c>
+      <c r="S175" s="88" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="176" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A176" s="8" t="s">
         <v>1108</v>
       </c>
-      <c r="B176" s="44" t="s">
+      <c r="B176" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C176" s="44" t="s">
-        <v>20</v>
-      </c>
-      <c r="D176" s="44" t="s">
-        <v>21</v>
-      </c>
-      <c r="E176" s="44"/>
-      <c r="F176" s="46" t="b">
-        <v>0</v>
-      </c>
-      <c r="G176" s="46"/>
-      <c r="H176" s="46" t="s">
-        <v>18</v>
-      </c>
-      <c r="I176" s="44" t="s">
-        <v>22</v>
-      </c>
-      <c r="J176" s="44" t="s">
-        <v>1249</v>
-      </c>
-      <c r="K176" s="44" t="s">
+      <c r="C176" s="41" t="s">
+        <v>1124</v>
+      </c>
+      <c r="D176" s="3" t="s">
+        <v>1127</v>
+      </c>
+      <c r="F176" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="G176" s="1" t="s">
+        <v>1211</v>
+      </c>
+      <c r="I176" s="3" t="s">
+        <v>1150</v>
+      </c>
+      <c r="J176" s="3" t="s">
+        <v>1247</v>
+      </c>
+      <c r="K176" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="L176" s="44" t="s">
+      <c r="L176" s="3" t="s">
         <v>1224</v>
       </c>
-      <c r="M176" s="44" t="s">
+      <c r="M176" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="N176" s="44" t="s">
+      <c r="N176" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="O176" s="44"/>
-      <c r="P176" s="47" t="s">
+      <c r="P176" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="Q176" s="62" t="s">
+      <c r="Q176" s="65" t="s">
         <v>26</v>
       </c>
-      <c r="R176" s="62" t="s">
+      <c r="R176" s="65" t="s">
         <v>26</v>
       </c>
-      <c r="S176" s="88" t="s">
+      <c r="S176" s="89" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="177" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="8" t="s">
         <v>1108</v>
       </c>
@@ -13438,46 +13441,37 @@
         <v>19</v>
       </c>
       <c r="C177" s="41" t="s">
-        <v>1124</v>
+        <v>1109</v>
       </c>
       <c r="D177" s="3" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="F177" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="G177" s="1" t="s">
-        <v>1211</v>
+        <v>0</v>
       </c>
       <c r="I177" s="3" t="s">
-        <v>1150</v>
-      </c>
-      <c r="J177" s="3" t="s">
-        <v>1247</v>
-      </c>
-      <c r="K177" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="L177" s="3" t="s">
-        <v>1224</v>
+        <v>1128</v>
+      </c>
+      <c r="J177" s="97" t="s">
+        <v>1170</v>
       </c>
       <c r="M177" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N177" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="P177" s="42" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q177" s="65" t="s">
-        <v>26</v>
-      </c>
-      <c r="R177" s="65" t="s">
-        <v>26</v>
-      </c>
-      <c r="S177" s="89" t="s">
-        <v>26</v>
+        <v>60</v>
+      </c>
+      <c r="P177" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q177" s="56" t="s">
+        <v>27</v>
+      </c>
+      <c r="R177" s="56" t="s">
+        <v>27</v>
+      </c>
+      <c r="S177" s="85" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="178" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -13488,37 +13482,43 @@
         <v>19</v>
       </c>
       <c r="C178" s="41" t="s">
-        <v>1109</v>
+        <v>531</v>
       </c>
       <c r="D178" s="3" t="s">
-        <v>1128</v>
+        <v>532</v>
       </c>
       <c r="F178" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="I178" s="3" t="s">
-        <v>1128</v>
-      </c>
-      <c r="J178" s="97" t="s">
-        <v>1170</v>
+      <c r="I178" s="41" t="s">
+        <v>1153</v>
+      </c>
+      <c r="J178" s="15" t="s">
+        <v>1240</v>
+      </c>
+      <c r="K178" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="L178" s="3" t="s">
+        <v>1233</v>
       </c>
       <c r="M178" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N178" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="P178" s="31" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q178" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="R178" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="S178" s="85" t="s">
-        <v>27</v>
+        <v>25</v>
+      </c>
+      <c r="P178" s="42" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q178" s="65" t="s">
+        <v>26</v>
+      </c>
+      <c r="R178" s="65" t="s">
+        <v>26</v>
+      </c>
+      <c r="S178" s="89" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="179" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -13529,25 +13529,19 @@
         <v>19</v>
       </c>
       <c r="C179" s="41" t="s">
-        <v>531</v>
+        <v>1112</v>
       </c>
       <c r="D179" s="3" t="s">
-        <v>532</v>
+        <v>1129</v>
       </c>
       <c r="F179" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I179" s="41" t="s">
-        <v>1153</v>
-      </c>
-      <c r="J179" s="15" t="s">
-        <v>1240</v>
-      </c>
-      <c r="K179" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="L179" s="3" t="s">
-        <v>1233</v>
+        <v>1154</v>
+      </c>
+      <c r="J179" s="93" t="s">
+        <v>1243</v>
       </c>
       <c r="M179" s="3" t="s">
         <v>24</v>
@@ -13555,17 +13549,17 @@
       <c r="N179" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="P179" s="42" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q179" s="65" t="s">
-        <v>26</v>
-      </c>
-      <c r="R179" s="65" t="s">
-        <v>26</v>
-      </c>
-      <c r="S179" s="89" t="s">
-        <v>26</v>
+      <c r="P179" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q179" s="56" t="s">
+        <v>27</v>
+      </c>
+      <c r="R179" s="56" t="s">
+        <v>27</v>
+      </c>
+      <c r="S179" s="85" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="180" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -13576,25 +13570,25 @@
         <v>19</v>
       </c>
       <c r="C180" s="41" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D180" s="3" t="s">
-        <v>1129</v>
+        <v>1113</v>
+      </c>
+      <c r="D180" s="17" t="s">
+        <v>1199</v>
       </c>
       <c r="F180" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I180" s="41" t="s">
-        <v>1154</v>
-      </c>
-      <c r="J180" s="93" t="s">
-        <v>1243</v>
+        <v>1155</v>
+      </c>
+      <c r="J180" s="68" t="s">
+        <v>1246</v>
       </c>
       <c r="M180" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N180" s="3" t="s">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="P180" s="31" t="s">
         <v>27</v>
@@ -13617,25 +13611,25 @@
         <v>19</v>
       </c>
       <c r="C181" s="41" t="s">
-        <v>1113</v>
-      </c>
-      <c r="D181" s="17" t="s">
-        <v>1199</v>
+        <v>1114</v>
+      </c>
+      <c r="D181" s="41" t="s">
+        <v>1131</v>
       </c>
       <c r="F181" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I181" s="41" t="s">
-        <v>1155</v>
-      </c>
-      <c r="J181" s="68" t="s">
-        <v>1246</v>
+        <v>1139</v>
+      </c>
+      <c r="J181" s="95" t="s">
+        <v>1245</v>
       </c>
       <c r="M181" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N181" s="3" t="s">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="P181" s="31" t="s">
         <v>27</v>
@@ -13658,25 +13652,25 @@
         <v>19</v>
       </c>
       <c r="C182" s="41" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="D182" s="41" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="F182" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I182" s="41" t="s">
-        <v>1139</v>
-      </c>
-      <c r="J182" s="95" t="s">
-        <v>1245</v>
+        <v>1140</v>
+      </c>
+      <c r="J182" s="68" t="s">
+        <v>1189</v>
       </c>
       <c r="M182" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="N182" s="3" t="s">
-        <v>25</v>
+      <c r="N182" t="s">
+        <v>60</v>
       </c>
       <c r="P182" s="31" t="s">
         <v>27</v>
@@ -13691,7 +13685,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="183" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="8" t="s">
         <v>1108</v>
       </c>
@@ -13699,25 +13693,25 @@
         <v>19</v>
       </c>
       <c r="C183" s="41" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="D183" s="41" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="F183" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I183" s="41" t="s">
-        <v>1140</v>
-      </c>
-      <c r="J183" s="68" t="s">
-        <v>1189</v>
+        <v>1141</v>
+      </c>
+      <c r="J183" s="94" t="s">
+        <v>1244</v>
       </c>
       <c r="M183" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="N183" t="s">
-        <v>60</v>
+      <c r="N183" s="3" t="s">
+        <v>25</v>
       </c>
       <c r="P183" s="31" t="s">
         <v>27</v>
@@ -13732,7 +13726,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="184" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" s="8" t="s">
         <v>1108</v>
       </c>
@@ -13740,20 +13734,18 @@
         <v>19</v>
       </c>
       <c r="C184" s="41" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="D184" s="41" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
       <c r="F184" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I184" s="41" t="s">
-        <v>1141</v>
-      </c>
-      <c r="J184" s="94" t="s">
-        <v>1244</v>
-      </c>
+        <v>1142</v>
+      </c>
+      <c r="J184" s="96"/>
       <c r="M184" s="3" t="s">
         <v>24</v>
       </c>
@@ -13773,7 +13765,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="185" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="8" t="s">
         <v>1108</v>
       </c>
@@ -13781,18 +13773,26 @@
         <v>19</v>
       </c>
       <c r="C185" s="41" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="D185" s="41" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
       <c r="F185" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I185" s="41" t="s">
-        <v>1142</v>
-      </c>
-      <c r="J185" s="96"/>
+        <v>1143</v>
+      </c>
+      <c r="J185" s="95">
+        <v>2.5</v>
+      </c>
+      <c r="K185" s="98" t="s">
+        <v>1257</v>
+      </c>
+      <c r="L185" t="s">
+        <v>1238</v>
+      </c>
       <c r="M185" s="3" t="s">
         <v>24</v>
       </c>
@@ -13812,7 +13812,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="186" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" s="8" t="s">
         <v>1108</v>
       </c>
@@ -13820,31 +13820,25 @@
         <v>19</v>
       </c>
       <c r="C186" s="41" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="D186" s="41" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="F186" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I186" s="41" t="s">
-        <v>1143</v>
-      </c>
-      <c r="J186" s="95">
-        <v>2.5</v>
-      </c>
-      <c r="K186" s="98" t="s">
-        <v>1257</v>
-      </c>
-      <c r="L186" t="s">
-        <v>1238</v>
+        <v>1144</v>
+      </c>
+      <c r="J186" s="33" t="s">
+        <v>1194</v>
       </c>
       <c r="M186" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N186" s="3" t="s">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="P186" s="31" t="s">
         <v>27</v>
@@ -13867,25 +13861,23 @@
         <v>19</v>
       </c>
       <c r="C187" s="41" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="D187" s="41" t="s">
-        <v>1136</v>
+        <v>1138</v>
       </c>
       <c r="F187" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I187" s="41" t="s">
-        <v>1144</v>
-      </c>
-      <c r="J187" s="33" t="s">
-        <v>1194</v>
-      </c>
+        <v>1145</v>
+      </c>
+      <c r="J187" s="96"/>
       <c r="M187" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N187" s="3" t="s">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="P187" s="31" t="s">
         <v>27</v>
@@ -13908,16 +13900,16 @@
         <v>19</v>
       </c>
       <c r="C188" s="41" t="s">
-        <v>1120</v>
+        <v>1121</v>
       </c>
       <c r="D188" s="41" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="F188" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I188" s="41" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="J188" s="96"/>
       <c r="M188" s="3" t="s">
@@ -13947,18 +13939,24 @@
         <v>19</v>
       </c>
       <c r="C189" s="41" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="D189" s="41" t="s">
-        <v>1137</v>
+        <v>1130</v>
       </c>
       <c r="F189" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I189" s="41" t="s">
-        <v>1146</v>
-      </c>
-      <c r="J189" s="96"/>
+        <v>1147</v>
+      </c>
+      <c r="J189" s="3"/>
+      <c r="K189" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="L189" s="3" t="s">
+        <v>1233</v>
+      </c>
       <c r="M189" s="3" t="s">
         <v>24</v>
       </c>
@@ -13978,7 +13976,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="190" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A190" s="8" t="s">
         <v>1108</v>
       </c>
@@ -13986,132 +13984,137 @@
         <v>19</v>
       </c>
       <c r="C190" s="41" t="s">
-        <v>1122</v>
+        <v>1123</v>
       </c>
       <c r="D190" s="41" t="s">
-        <v>1130</v>
+        <v>1148</v>
       </c>
       <c r="F190" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I190" s="41" t="s">
-        <v>1147</v>
+        <v>1149</v>
       </c>
       <c r="J190" s="3"/>
-      <c r="K190" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="L190" s="3" t="s">
-        <v>1233</v>
-      </c>
       <c r="M190" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N190" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="P190" s="31" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q190" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="R190" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="S190" s="85" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="191" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A191" s="8" t="s">
-        <v>1108</v>
-      </c>
-      <c r="B191" s="3" t="s">
+      <c r="P190" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q190" s="57" t="s">
+        <v>27</v>
+      </c>
+      <c r="R190" s="57" t="s">
+        <v>27</v>
+      </c>
+      <c r="S190" s="86" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="191" spans="1:19" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A191" s="48" t="s">
+        <v>711</v>
+      </c>
+      <c r="B191" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="C191" s="41" t="s">
-        <v>1123</v>
-      </c>
-      <c r="D191" s="41" t="s">
-        <v>1148</v>
-      </c>
-      <c r="F191" s="1" t="b">
+      <c r="C191" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="D191" s="48" t="s">
+        <v>21</v>
+      </c>
+      <c r="E191" s="44"/>
+      <c r="F191" s="46" t="b">
         <v>0</v>
       </c>
-      <c r="I191" s="41" t="s">
-        <v>1149</v>
-      </c>
-      <c r="J191" s="3"/>
-      <c r="M191" s="3" t="s">
+      <c r="G191" s="46"/>
+      <c r="H191" s="46" t="s">
+        <v>18</v>
+      </c>
+      <c r="I191" s="44" t="s">
+        <v>22</v>
+      </c>
+      <c r="J191" s="44" t="s">
+        <v>1249</v>
+      </c>
+      <c r="K191" s="44" t="s">
+        <v>23</v>
+      </c>
+      <c r="L191" s="44" t="s">
+        <v>1224</v>
+      </c>
+      <c r="M191" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="N191" s="3" t="s">
+      <c r="N191" s="44" t="s">
         <v>25</v>
       </c>
-      <c r="P191" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q191" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="R191" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="S191" s="86" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="192" spans="1:19" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A192" s="48" t="s">
+      <c r="O191" s="48"/>
+      <c r="P191" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q191" s="62" t="s">
+        <v>26</v>
+      </c>
+      <c r="R191" s="62" t="s">
+        <v>26</v>
+      </c>
+      <c r="S191" s="88" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="192" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A192" t="s">
         <v>711</v>
       </c>
-      <c r="B192" s="48" t="s">
+      <c r="B192" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C192" s="48" t="s">
-        <v>20</v>
-      </c>
-      <c r="D192" s="48" t="s">
-        <v>21</v>
-      </c>
-      <c r="E192" s="44"/>
-      <c r="F192" s="46" t="b">
-        <v>0</v>
-      </c>
-      <c r="G192" s="46"/>
-      <c r="H192" s="46" t="s">
-        <v>18</v>
-      </c>
-      <c r="I192" s="44" t="s">
-        <v>22</v>
-      </c>
-      <c r="J192" s="44" t="s">
-        <v>1249</v>
-      </c>
-      <c r="K192" s="44" t="s">
+      <c r="C192" t="s">
+        <v>1099</v>
+      </c>
+      <c r="D192" t="s">
+        <v>682</v>
+      </c>
+      <c r="F192" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="G192" s="1" t="s">
+        <v>1212</v>
+      </c>
+      <c r="I192" s="3" t="s">
+        <v>1157</v>
+      </c>
+      <c r="J192" s="3" t="s">
+        <v>1255</v>
+      </c>
+      <c r="K192" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="L192" s="44" t="s">
+      <c r="L192" s="3" t="s">
         <v>1224</v>
       </c>
-      <c r="M192" s="44" t="s">
+      <c r="M192" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="N192" s="44" t="s">
+      <c r="N192" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="O192" s="48"/>
-      <c r="P192" s="47" t="s">
+      <c r="P192" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="Q192" s="62" t="s">
+      <c r="Q192" s="65" t="s">
         <v>26</v>
       </c>
-      <c r="R192" s="62" t="s">
+      <c r="R192" s="65" t="s">
         <v>26</v>
       </c>
-      <c r="S192" s="88" t="s">
+      <c r="S192" s="89" t="s">
         <v>26</v>
       </c>
     </row>
@@ -14122,23 +14125,23 @@
       <c r="B193" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C193" t="s">
-        <v>1099</v>
-      </c>
-      <c r="D193" t="s">
-        <v>682</v>
+      <c r="C193" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="D193" s="3" t="s">
+        <v>279</v>
       </c>
       <c r="F193" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="G193" s="1" t="s">
-        <v>1212</v>
+        <v>0</v>
+      </c>
+      <c r="H193" s="1" t="s">
+        <v>277</v>
       </c>
       <c r="I193" s="3" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="J193" s="3" t="s">
-        <v>1255</v>
+        <v>1252</v>
       </c>
       <c r="K193" s="3" t="s">
         <v>23</v>
@@ -14172,23 +14175,23 @@
       <c r="B194" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C194" s="3" t="s">
-        <v>278</v>
+      <c r="C194" t="s">
+        <v>1100</v>
       </c>
       <c r="D194" s="3" t="s">
-        <v>279</v>
+        <v>1127</v>
       </c>
       <c r="F194" s="1" t="b">
         <v>0</v>
       </c>
       <c r="H194" s="1" t="s">
-        <v>277</v>
+        <v>1108</v>
       </c>
       <c r="I194" s="3" t="s">
-        <v>1156</v>
+        <v>1150</v>
       </c>
       <c r="J194" s="3" t="s">
-        <v>1252</v>
+        <v>1247</v>
       </c>
       <c r="K194" s="3" t="s">
         <v>23</v>
@@ -14223,34 +14226,25 @@
         <v>19</v>
       </c>
       <c r="C195" t="s">
-        <v>1100</v>
+        <v>711</v>
       </c>
       <c r="D195" s="3" t="s">
-        <v>1127</v>
+        <v>710</v>
       </c>
       <c r="F195" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H195" s="1" t="s">
-        <v>1108</v>
-      </c>
       <c r="I195" s="3" t="s">
-        <v>1150</v>
+        <v>1158</v>
       </c>
       <c r="J195" s="3" t="s">
-        <v>1247</v>
-      </c>
-      <c r="K195" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="L195" s="3" t="s">
-        <v>1224</v>
+        <v>1256</v>
       </c>
       <c r="M195" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="N195" s="3" t="s">
-        <v>25</v>
+      <c r="N195" t="s">
+        <v>519</v>
       </c>
       <c r="P195" s="42" t="s">
         <v>26</v>
@@ -14273,25 +14267,32 @@
         <v>19</v>
       </c>
       <c r="C196" t="s">
-        <v>711</v>
+        <v>1200</v>
       </c>
       <c r="D196" s="3" t="s">
-        <v>710</v>
-      </c>
-      <c r="F196" s="1" t="b">
+        <v>1169</v>
+      </c>
+      <c r="F196" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I196" s="3" t="s">
-        <v>1158</v>
-      </c>
-      <c r="J196" s="3" t="s">
-        <v>1256</v>
+      <c r="G196" s="43"/>
+      <c r="I196" s="41" t="s">
+        <v>1162</v>
+      </c>
+      <c r="J196" s="93" t="s">
+        <v>1254</v>
+      </c>
+      <c r="K196" s="3" t="s">
+        <v>1213</v>
+      </c>
+      <c r="L196" s="3" t="s">
+        <v>1237</v>
       </c>
       <c r="M196" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="N196" t="s">
-        <v>519</v>
+      <c r="N196" s="3" t="s">
+        <v>25</v>
       </c>
       <c r="P196" s="42" t="s">
         <v>26</v>
@@ -14313,33 +14314,27 @@
       <c r="B197" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C197" t="s">
-        <v>1200</v>
+      <c r="C197" s="41" t="s">
+        <v>1159</v>
       </c>
       <c r="D197" s="3" t="s">
-        <v>1169</v>
+        <v>1164</v>
       </c>
       <c r="F197" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G197" s="43"/>
-      <c r="I197" s="41" t="s">
-        <v>1162</v>
-      </c>
-      <c r="J197" s="93" t="s">
-        <v>1254</v>
-      </c>
-      <c r="K197" s="3" t="s">
-        <v>1213</v>
-      </c>
-      <c r="L197" s="3" t="s">
-        <v>1237</v>
+      <c r="I197" s="3" t="s">
+        <v>1160</v>
+      </c>
+      <c r="J197" s="68" t="s">
+        <v>1180</v>
       </c>
       <c r="M197" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="N197" s="3" t="s">
-        <v>25</v>
+      <c r="N197" t="s">
+        <v>60</v>
       </c>
       <c r="P197" s="42" t="s">
         <v>26</v>
@@ -14362,38 +14357,44 @@
         <v>19</v>
       </c>
       <c r="C198" s="41" t="s">
-        <v>1159</v>
-      </c>
-      <c r="D198" s="3" t="s">
-        <v>1164</v>
+        <v>1110</v>
+      </c>
+      <c r="D198" s="41" t="s">
+        <v>1165</v>
       </c>
       <c r="F198" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G198" s="43"/>
-      <c r="I198" s="3" t="s">
-        <v>1160</v>
-      </c>
-      <c r="J198" s="68" t="s">
-        <v>1180</v>
+      <c r="I198" s="41" t="s">
+        <v>1151</v>
+      </c>
+      <c r="J198" s="3">
+        <v>4</v>
+      </c>
+      <c r="K198" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="L198" t="s">
+        <v>1231</v>
       </c>
       <c r="M198" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="N198" t="s">
-        <v>60</v>
-      </c>
-      <c r="P198" s="42" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q198" s="65" t="s">
-        <v>26</v>
-      </c>
-      <c r="R198" s="65" t="s">
-        <v>26</v>
-      </c>
-      <c r="S198" s="89" t="s">
-        <v>26</v>
+      <c r="N198" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="P198" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q198" s="56" t="s">
+        <v>27</v>
+      </c>
+      <c r="R198" s="56" t="s">
+        <v>27</v>
+      </c>
+      <c r="S198" s="85" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="199" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -14404,20 +14405,20 @@
         <v>19</v>
       </c>
       <c r="C199" s="41" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="D199" s="41" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="F199" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G199" s="43"/>
       <c r="I199" s="41" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="J199" s="3">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="K199" s="3" t="s">
         <v>241</v>
@@ -14452,20 +14453,20 @@
         <v>19</v>
       </c>
       <c r="C200" s="41" t="s">
-        <v>1111</v>
+        <v>1125</v>
       </c>
       <c r="D200" s="41" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="F200" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G200" s="43"/>
       <c r="I200" s="41" t="s">
-        <v>1152</v>
+        <v>1161</v>
       </c>
       <c r="J200" s="3">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="K200" s="3" t="s">
         <v>241</v>
@@ -14500,26 +14501,26 @@
         <v>19</v>
       </c>
       <c r="C201" s="41" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="D201" s="41" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="F201" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G201" s="43"/>
       <c r="I201" s="41" t="s">
-        <v>1161</v>
-      </c>
-      <c r="J201" s="3">
-        <v>90</v>
+        <v>1163</v>
+      </c>
+      <c r="J201" s="3" t="s">
+        <v>53</v>
       </c>
       <c r="K201" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="L201" t="s">
-        <v>1231</v>
+        <v>54</v>
+      </c>
+      <c r="L201" s="3" t="s">
+        <v>1225</v>
       </c>
       <c r="M201" s="3" t="s">
         <v>24</v>
@@ -14541,60 +14542,12 @@
       </c>
     </row>
     <row r="202" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A202" t="s">
-        <v>711</v>
-      </c>
-      <c r="B202" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C202" s="41" t="s">
-        <v>1126</v>
-      </c>
-      <c r="D202" s="41" t="s">
-        <v>1168</v>
-      </c>
-      <c r="F202" s="43" t="b">
-        <v>0</v>
-      </c>
-      <c r="G202" s="43"/>
-      <c r="I202" s="41" t="s">
-        <v>1163</v>
-      </c>
-      <c r="J202" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="K202" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="L202" s="3" t="s">
-        <v>1225</v>
-      </c>
-      <c r="M202" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="N202" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="P202" s="31" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q202" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="R202" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="S202" s="85" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="203" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J203" s="3"/>
+      <c r="J202" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S202" xr:uid="{545CA0C1-0282-3A43-9C60-512DE414A571}"/>
+  <autoFilter ref="A1:S201" xr:uid="{545CA0C1-0282-3A43-9C60-512DE414A571}"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S26:S30 S172 P2:R202" xr:uid="{D3C8CE10-E7EB-B24A-855C-B8189CB5A06C}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S26:S30 S171 P2:R201" xr:uid="{D3C8CE10-E7EB-B24A-855C-B8189CB5A06C}"/>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="O3" r:id="rId1" xr:uid="{4D6B5FE8-0E6D-E84F-B3F9-D5B11E30DF9B}"/>
@@ -14655,7 +14608,7 @@
     <hyperlink ref="J39" r:id="rId56" xr:uid="{641DCDA6-12A3-44F1-96D1-1EACA7591B2E}"/>
     <hyperlink ref="O30" r:id="rId57" xr:uid="{2BA242DC-2C53-4118-835C-02CD479C61F0}"/>
     <hyperlink ref="O43" r:id="rId58" display="http://purl.obolibrary.org/obo/CL_0000000" xr:uid="{332E6129-6494-114C-9111-B9D6271B6C6D}"/>
-    <hyperlink ref="J179" r:id="rId59" xr:uid="{36FAB4CA-D2E7-2648-850A-DCF88860F33D}"/>
+    <hyperlink ref="J178" r:id="rId59" xr:uid="{36FAB4CA-D2E7-2648-850A-DCF88860F33D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId60"/>

</xml_diff>

<commit_message>
CD-182: Remove duplicate word "Sequencing" from technology name in "technologies" work sheet
</commit_message>
<xml_diff>
--- a/single_cell/singlecell_schema_main_v0.4.xlsx
+++ b/single_cell/singlecell_schema_main_v0.4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zef22hak/development/COPO-schemas/single_cell/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/providen/Documents/EI/Projects/COPO-schemas/single_cell/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A716B4C-E7AD-5149-A9F8-6706772BBE40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{118AE7D9-7D3B-BE48-BB38-532C475A47CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
+    <workbookView xWindow="31760" yWindow="340" windowWidth="30240" windowHeight="18080" activeTab="7" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3123" uniqueCount="1267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3121" uniqueCount="1265">
   <si>
     <t>component_name</t>
   </si>
@@ -2912,9 +2912,6 @@
   </si>
   <si>
     <t>sc_rnaseq</t>
-  </si>
-  <si>
-    <t>stx_seq</t>
   </si>
   <si>
     <t>repository_ena</t>
@@ -3409,12 +3406,6 @@
   </si>
   <si>
     <t>Functional Annotation of Animal Genomes (FAANG)</t>
-  </si>
-  <si>
-    <t>Single-cell Ribonucleic Acid Sequencing Sequencing (scRNA-Seq)</t>
-  </si>
-  <si>
-    <t>Spatial Transcriptomics Sequencing (ST-Seq)</t>
   </si>
   <si>
     <t>ENA</t>
@@ -4014,6 +4005,9 @@
   </si>
   <si>
     <t>A unique reference or identifier for the sample. This field must provide a consistent, unambiguous way to identify the sample within and across datasets. It can be a name, code, or accession-like format, as long as it remains unique.</t>
+  </si>
+  <si>
+    <t>Single-cell Ribonucleic Acid Sequencing (scRNA-Seq)</t>
   </si>
 </sst>
 </file>
@@ -5421,7 +5415,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>6</v>
@@ -5480,13 +5474,13 @@
         <v>22</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>24</v>
@@ -5714,7 +5708,7 @@
         <v>54</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>1225</v>
+        <v>1222</v>
       </c>
       <c r="M7" s="3" t="s">
         <v>24</v>
@@ -5887,7 +5881,7 @@
         <v>23</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M11" s="3" t="s">
         <v>24</v>
@@ -5928,10 +5922,10 @@
         <v>79</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>1259</v>
+        <v>1256</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>1261</v>
+        <v>1258</v>
       </c>
       <c r="M12" s="3" t="s">
         <v>81</v>
@@ -5975,7 +5969,7 @@
         <v>87</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="M13" s="3" t="s">
         <v>24</v>
@@ -6057,7 +6051,7 @@
         <v>98</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>1227</v>
+        <v>1224</v>
       </c>
       <c r="M15" s="3" t="s">
         <v>24</v>
@@ -6134,7 +6128,7 @@
         <v>104</v>
       </c>
       <c r="J17" t="s">
-        <v>1106</v>
+        <v>1103</v>
       </c>
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
@@ -6183,13 +6177,13 @@
         <v>22</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M18" s="2" t="s">
         <v>24</v>
@@ -6237,7 +6231,7 @@
         <v>111</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>1228</v>
+        <v>1225</v>
       </c>
       <c r="M19" s="3" t="s">
         <v>24</v>
@@ -6285,7 +6279,7 @@
         <v>117</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="M20" s="3" t="s">
         <v>24</v>
@@ -6335,7 +6329,7 @@
         <v>123</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>24</v>
@@ -6385,7 +6379,7 @@
         <v>129</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>1229</v>
+        <v>1226</v>
       </c>
       <c r="M22" s="3" t="s">
         <v>24</v>
@@ -6435,7 +6429,7 @@
         <v>135</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="M23" s="3" t="s">
         <v>24</v>
@@ -6531,7 +6525,7 @@
         <v>146</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>24</v>
@@ -6580,13 +6574,13 @@
         <v>149</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="K26" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M26" s="2" t="s">
         <v>24</v>
@@ -6625,10 +6619,10 @@
         <v>1</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>1266</v>
+        <v>1263</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>1251</v>
+        <v>1248</v>
       </c>
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
@@ -6657,7 +6651,7 @@
         <v>148</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>152</v>
@@ -6681,7 +6675,7 @@
         <v>135</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>1230</v>
+        <v>1227</v>
       </c>
       <c r="M28" s="3" t="s">
         <v>24</v>
@@ -6710,7 +6704,7 @@
         <v>148</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>159</v>
@@ -6734,7 +6728,7 @@
         <v>162</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M29" s="3" t="s">
         <v>24</v>
@@ -6763,7 +6757,7 @@
         <v>148</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>164</v>
@@ -6832,13 +6826,13 @@
         <v>22</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="K31" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M31" s="2" t="s">
         <v>24</v>
@@ -6877,19 +6871,19 @@
         <v>1</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>1206</v>
+        <v>1203</v>
       </c>
       <c r="I32" s="3" t="s">
         <v>173</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>1248</v>
+        <v>1245</v>
       </c>
       <c r="K32" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M32" s="3" t="s">
         <v>24</v>
@@ -7143,7 +7137,7 @@
         <v>193</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>1260</v>
+        <v>1257</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>194</v>
@@ -7161,7 +7155,7 @@
         <v>87</v>
       </c>
       <c r="L38" s="3" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="M38" s="3" t="s">
         <v>24</v>
@@ -7212,7 +7206,7 @@
         <v>201</v>
       </c>
       <c r="L39" s="3" t="s">
-        <v>1233</v>
+        <v>1230</v>
       </c>
       <c r="M39" s="3" t="s">
         <v>24</v>
@@ -7380,22 +7374,22 @@
         <v>216</v>
       </c>
       <c r="J43" s="17" t="s">
-        <v>1223</v>
+        <v>1220</v>
       </c>
       <c r="K43" s="3" t="s">
         <v>217</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="M43" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N43" s="92" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="O43" s="13" t="s">
-        <v>1204</v>
+        <v>1201</v>
       </c>
       <c r="P43" s="31"/>
       <c r="Q43" s="56"/>
@@ -7471,7 +7465,7 @@
         <v>225</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="M45" s="3" t="s">
         <v>24</v>
@@ -7512,13 +7506,13 @@
         <v>22</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="K46" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>1232</v>
+        <v>1229</v>
       </c>
       <c r="M46" s="2" t="s">
         <v>24</v>
@@ -7557,19 +7551,19 @@
         <v>1</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>1207</v>
+        <v>1204</v>
       </c>
       <c r="I47" s="3" t="s">
         <v>229</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>1250</v>
+        <v>1247</v>
       </c>
       <c r="K47" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L47" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M47" s="3" t="s">
         <v>24</v>
@@ -7611,10 +7605,10 @@
         <v>148</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>1264</v>
+        <v>1261</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>1251</v>
+        <v>1248</v>
       </c>
       <c r="K48" s="3"/>
       <c r="L48" s="3"/>
@@ -7661,13 +7655,13 @@
         <v>173</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>1248</v>
+        <v>1245</v>
       </c>
       <c r="K49" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L49" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M49" s="3" t="s">
         <v>24</v>
@@ -7757,7 +7751,7 @@
         <v>201</v>
       </c>
       <c r="L51" t="s">
-        <v>1233</v>
+        <v>1230</v>
       </c>
       <c r="M51" s="3" t="s">
         <v>24</v>
@@ -7802,7 +7796,7 @@
         <v>241</v>
       </c>
       <c r="L52" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M52" s="3" t="s">
         <v>24</v>
@@ -8157,7 +8151,7 @@
         <v>241</v>
       </c>
       <c r="L60" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M60" s="3" t="s">
         <v>24</v>
@@ -8249,7 +8243,7 @@
         <v>225</v>
       </c>
       <c r="L62" s="3" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="M62" s="3" t="s">
         <v>24</v>
@@ -8290,13 +8284,13 @@
         <v>22</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="K63" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M63" s="2" t="s">
         <v>24</v>
@@ -8335,19 +8329,19 @@
         <v>1</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>1208</v>
+        <v>1205</v>
       </c>
       <c r="I64" s="3" t="s">
         <v>280</v>
       </c>
       <c r="J64" s="3" t="s">
-        <v>1252</v>
+        <v>1249</v>
       </c>
       <c r="K64" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L64" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M64" s="3" t="s">
         <v>24</v>
@@ -8392,13 +8386,13 @@
         <v>281</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>1250</v>
+        <v>1247</v>
       </c>
       <c r="K65" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L65" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M65" s="3" t="s">
         <v>24</v>
@@ -8440,10 +8434,10 @@
         <v>148</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>1265</v>
+        <v>1262</v>
       </c>
       <c r="J66" s="3" t="s">
-        <v>1251</v>
+        <v>1248</v>
       </c>
       <c r="K66" s="3"/>
       <c r="L66" s="3"/>
@@ -8510,7 +8504,7 @@
         <v>277</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="C68" s="3" t="s">
         <v>287</v>
@@ -8531,7 +8525,7 @@
         <v>241</v>
       </c>
       <c r="L68" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M68" s="3" t="s">
         <v>24</v>
@@ -8628,7 +8622,7 @@
         <v>241</v>
       </c>
       <c r="L70" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M70" s="3" t="s">
         <v>24</v>
@@ -8676,7 +8670,7 @@
         <v>241</v>
       </c>
       <c r="L71" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M71" s="3" t="s">
         <v>24</v>
@@ -9334,13 +9328,13 @@
         <v>362</v>
       </c>
       <c r="J86" s="3" t="s">
-        <v>1258</v>
+        <v>1255</v>
       </c>
       <c r="K86" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L86" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M86" s="3" t="s">
         <v>24</v>
@@ -9432,7 +9426,7 @@
         <v>241</v>
       </c>
       <c r="L88" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M88" s="3" t="s">
         <v>24</v>
@@ -9527,7 +9521,7 @@
         <v>379</v>
       </c>
       <c r="L90" t="s">
-        <v>1236</v>
+        <v>1233</v>
       </c>
       <c r="M90" s="3" t="s">
         <v>24</v>
@@ -9571,7 +9565,7 @@
         <v>379</v>
       </c>
       <c r="L91" t="s">
-        <v>1236</v>
+        <v>1233</v>
       </c>
       <c r="M91" s="3" t="s">
         <v>24</v>
@@ -9615,7 +9609,7 @@
         <v>390</v>
       </c>
       <c r="L92" s="3" t="s">
-        <v>1239</v>
+        <v>1236</v>
       </c>
       <c r="M92" s="3" t="s">
         <v>24</v>
@@ -9699,7 +9693,7 @@
         <v>400</v>
       </c>
       <c r="L94" s="3" t="s">
-        <v>1235</v>
+        <v>1232</v>
       </c>
       <c r="M94" s="3" t="s">
         <v>24</v>
@@ -9857,13 +9851,13 @@
         <v>419</v>
       </c>
       <c r="J98" s="91" t="s">
-        <v>1222</v>
+        <v>1219</v>
       </c>
       <c r="K98" s="3" t="s">
         <v>54</v>
       </c>
       <c r="L98" s="3" t="s">
-        <v>1225</v>
+        <v>1222</v>
       </c>
       <c r="M98" s="3" t="s">
         <v>24</v>
@@ -9902,7 +9896,7 @@
         <v>201</v>
       </c>
       <c r="L99" s="3" t="s">
-        <v>1233</v>
+        <v>1230</v>
       </c>
       <c r="M99" s="3" t="s">
         <v>24</v>
@@ -10125,13 +10119,13 @@
         <v>22</v>
       </c>
       <c r="J104" s="2" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="K104" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L104" s="2" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M104" s="2" t="s">
         <v>24</v>
@@ -10158,7 +10152,7 @@
         <v>435</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="C105" s="3" t="s">
         <v>436</v>
@@ -10170,19 +10164,19 @@
         <v>1</v>
       </c>
       <c r="G105" s="1" t="s">
-        <v>1209</v>
+        <v>1206</v>
       </c>
       <c r="I105" s="3" t="s">
         <v>438</v>
       </c>
       <c r="J105" s="3" t="s">
-        <v>1253</v>
+        <v>1250</v>
       </c>
       <c r="K105" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L105" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M105" s="3" t="s">
         <v>24</v>
@@ -10211,7 +10205,7 @@
         <v>435</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="C106" s="3" t="s">
         <v>440</v>
@@ -10257,7 +10251,7 @@
         <v>435</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="C107" s="3" t="s">
         <v>445</v>
@@ -10420,7 +10414,7 @@
         <v>241</v>
       </c>
       <c r="L110" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M110" s="3" t="s">
         <v>24</v>
@@ -10468,7 +10462,7 @@
         <v>241</v>
       </c>
       <c r="L111" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M111" s="3" t="s">
         <v>24</v>
@@ -10495,7 +10489,7 @@
         <v>435</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="C112" s="3" t="s">
         <v>467</v>
@@ -10541,7 +10535,7 @@
         <v>435</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="C113" s="3" t="s">
         <v>472</v>
@@ -10562,7 +10556,7 @@
         <v>241</v>
       </c>
       <c r="L113" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M113" s="3" t="s">
         <v>24</v>
@@ -10591,7 +10585,7 @@
         <v>435</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="C114" s="3" t="s">
         <v>476</v>
@@ -10612,7 +10606,7 @@
         <v>241</v>
       </c>
       <c r="L114" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M114" s="3" t="s">
         <v>24</v>
@@ -10641,7 +10635,7 @@
         <v>435</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="C115" s="3" t="s">
         <v>479</v>
@@ -10687,7 +10681,7 @@
         <v>435</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="C116" s="3" t="s">
         <v>484</v>
@@ -10708,7 +10702,7 @@
         <v>241</v>
       </c>
       <c r="L116" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M116" s="3" t="s">
         <v>24</v>
@@ -10737,7 +10731,7 @@
         <v>435</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="C117" s="3" t="s">
         <v>488</v>
@@ -10758,7 +10752,7 @@
         <v>241</v>
       </c>
       <c r="L117" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M117" s="3" t="s">
         <v>24</v>
@@ -10808,7 +10802,7 @@
         <v>241</v>
       </c>
       <c r="L118" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M118" s="3" t="s">
         <v>24</v>
@@ -10892,7 +10886,7 @@
         <v>241</v>
       </c>
       <c r="L120" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M120" s="3" t="s">
         <v>24</v>
@@ -10976,7 +10970,7 @@
         <v>241</v>
       </c>
       <c r="L122" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M122" s="3" t="s">
         <v>24</v>
@@ -11019,13 +11013,13 @@
         <v>22</v>
       </c>
       <c r="J123" s="2" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="K123" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L123" s="2" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M123" s="2" t="s">
         <v>24</v>
@@ -11248,13 +11242,13 @@
         <v>22</v>
       </c>
       <c r="J128" s="2" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="K128" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L128" s="2" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M128" s="2" t="s">
         <v>24</v>
@@ -11958,7 +11952,7 @@
         <v>241</v>
       </c>
       <c r="L144" s="3" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M144" s="3" t="s">
         <v>24</v>
@@ -12122,7 +12116,7 @@
         <v>614</v>
       </c>
       <c r="L148" s="3" t="s">
-        <v>1234</v>
+        <v>1231</v>
       </c>
       <c r="M148" s="3" t="s">
         <v>24</v>
@@ -12206,7 +12200,7 @@
         <v>614</v>
       </c>
       <c r="L150" s="3" t="s">
-        <v>1234</v>
+        <v>1231</v>
       </c>
       <c r="M150" s="3" t="s">
         <v>24</v>
@@ -12289,13 +12283,13 @@
         <v>22</v>
       </c>
       <c r="J152" s="2" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="K152" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L152" s="2" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M152" s="2" t="s">
         <v>24</v>
@@ -12566,7 +12560,7 @@
         <v>23</v>
       </c>
       <c r="L158" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M158" s="3" t="s">
         <v>24</v>
@@ -12833,13 +12827,13 @@
         <v>22</v>
       </c>
       <c r="J164" s="2" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="K164" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L164" s="2" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M164" s="2" t="s">
         <v>24</v>
@@ -12878,19 +12872,19 @@
         <v>1</v>
       </c>
       <c r="G165" s="1" t="s">
-        <v>1210</v>
+        <v>1207</v>
       </c>
       <c r="I165" s="3" t="s">
         <v>683</v>
       </c>
       <c r="J165" s="3" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="K165" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L165" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M165" s="3" t="s">
         <v>24</v>
@@ -12935,13 +12929,13 @@
         <v>280</v>
       </c>
       <c r="J166" s="3" t="s">
-        <v>1252</v>
+        <v>1249</v>
       </c>
       <c r="K166" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L166" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M166" s="3" t="s">
         <v>24</v>
@@ -12986,13 +12980,13 @@
         <v>438</v>
       </c>
       <c r="J167" s="3" t="s">
-        <v>1253</v>
+        <v>1250</v>
       </c>
       <c r="K167" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L167" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M167" s="3" t="s">
         <v>24</v>
@@ -13210,13 +13204,13 @@
         <v>702</v>
       </c>
       <c r="J172" s="41" t="s">
-        <v>1242</v>
+        <v>1239</v>
       </c>
       <c r="K172" s="3" t="s">
-        <v>1213</v>
+        <v>1210</v>
       </c>
       <c r="L172" s="3" t="s">
-        <v>1237</v>
+        <v>1234</v>
       </c>
       <c r="M172" s="3" t="s">
         <v>24</v>
@@ -13258,13 +13252,13 @@
         <v>705</v>
       </c>
       <c r="J173" s="93" t="s">
-        <v>1241</v>
+        <v>1238</v>
       </c>
       <c r="K173" s="3" t="s">
-        <v>1213</v>
+        <v>1210</v>
       </c>
       <c r="L173" s="3" t="s">
-        <v>1237</v>
+        <v>1234</v>
       </c>
       <c r="M173" s="3" t="s">
         <v>24</v>
@@ -13332,7 +13326,7 @@
     </row>
     <row r="175" spans="1:19" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A175" s="45" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B175" s="44" t="s">
         <v>19</v>
@@ -13355,13 +13349,13 @@
         <v>22</v>
       </c>
       <c r="J175" s="44" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="K175" s="44" t="s">
         <v>23</v>
       </c>
       <c r="L175" s="44" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M175" s="44" t="s">
         <v>24</v>
@@ -13385,34 +13379,34 @@
     </row>
     <row r="176" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A176" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B176" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C176" s="41" t="s">
+        <v>1121</v>
+      </c>
+      <c r="D176" s="3" t="s">
         <v>1124</v>
-      </c>
-      <c r="D176" s="3" t="s">
-        <v>1127</v>
       </c>
       <c r="F176" s="1" t="b">
         <v>1</v>
       </c>
       <c r="G176" s="1" t="s">
-        <v>1211</v>
+        <v>1208</v>
       </c>
       <c r="I176" s="3" t="s">
-        <v>1150</v>
+        <v>1147</v>
       </c>
       <c r="J176" s="3" t="s">
-        <v>1247</v>
+        <v>1244</v>
       </c>
       <c r="K176" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L176" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M176" s="3" t="s">
         <v>24</v>
@@ -13435,25 +13429,25 @@
     </row>
     <row r="177" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B177" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C177" s="41" t="s">
-        <v>1109</v>
+        <v>1106</v>
       </c>
       <c r="D177" s="3" t="s">
-        <v>1128</v>
+        <v>1125</v>
       </c>
       <c r="F177" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I177" s="3" t="s">
-        <v>1128</v>
+        <v>1125</v>
       </c>
       <c r="J177" s="97" t="s">
-        <v>1170</v>
+        <v>1167</v>
       </c>
       <c r="M177" s="3" t="s">
         <v>24</v>
@@ -13476,7 +13470,7 @@
     </row>
     <row r="178" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B178" s="3" t="s">
         <v>19</v>
@@ -13491,16 +13485,16 @@
         <v>0</v>
       </c>
       <c r="I178" s="41" t="s">
-        <v>1153</v>
+        <v>1150</v>
       </c>
       <c r="J178" s="15" t="s">
-        <v>1240</v>
+        <v>1237</v>
       </c>
       <c r="K178" s="3" t="s">
         <v>201</v>
       </c>
       <c r="L178" s="3" t="s">
-        <v>1233</v>
+        <v>1230</v>
       </c>
       <c r="M178" s="3" t="s">
         <v>24</v>
@@ -13523,25 +13517,25 @@
     </row>
     <row r="179" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B179" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C179" s="41" t="s">
-        <v>1112</v>
+        <v>1109</v>
       </c>
       <c r="D179" s="3" t="s">
-        <v>1129</v>
+        <v>1126</v>
       </c>
       <c r="F179" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I179" s="41" t="s">
-        <v>1154</v>
+        <v>1151</v>
       </c>
       <c r="J179" s="93" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
       <c r="M179" s="3" t="s">
         <v>24</v>
@@ -13564,25 +13558,25 @@
     </row>
     <row r="180" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B180" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C180" s="41" t="s">
-        <v>1113</v>
+        <v>1110</v>
       </c>
       <c r="D180" s="17" t="s">
-        <v>1199</v>
+        <v>1196</v>
       </c>
       <c r="F180" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I180" s="41" t="s">
-        <v>1155</v>
+        <v>1152</v>
       </c>
       <c r="J180" s="68" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="M180" s="3" t="s">
         <v>24</v>
@@ -13605,25 +13599,25 @@
     </row>
     <row r="181" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B181" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C181" s="41" t="s">
-        <v>1114</v>
+        <v>1111</v>
       </c>
       <c r="D181" s="41" t="s">
-        <v>1131</v>
+        <v>1128</v>
       </c>
       <c r="F181" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I181" s="41" t="s">
-        <v>1139</v>
+        <v>1136</v>
       </c>
       <c r="J181" s="95" t="s">
-        <v>1245</v>
+        <v>1242</v>
       </c>
       <c r="M181" s="3" t="s">
         <v>24</v>
@@ -13646,25 +13640,25 @@
     </row>
     <row r="182" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B182" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C182" s="41" t="s">
-        <v>1115</v>
+        <v>1112</v>
       </c>
       <c r="D182" s="41" t="s">
-        <v>1132</v>
+        <v>1129</v>
       </c>
       <c r="F182" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I182" s="41" t="s">
-        <v>1140</v>
+        <v>1137</v>
       </c>
       <c r="J182" s="68" t="s">
-        <v>1189</v>
+        <v>1186</v>
       </c>
       <c r="M182" s="3" t="s">
         <v>24</v>
@@ -13687,25 +13681,25 @@
     </row>
     <row r="183" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B183" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C183" s="41" t="s">
-        <v>1116</v>
+        <v>1113</v>
       </c>
       <c r="D183" s="41" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="F183" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I183" s="41" t="s">
-        <v>1141</v>
+        <v>1138</v>
       </c>
       <c r="J183" s="94" t="s">
-        <v>1244</v>
+        <v>1241</v>
       </c>
       <c r="M183" s="3" t="s">
         <v>24</v>
@@ -13728,22 +13722,22 @@
     </row>
     <row r="184" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B184" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C184" s="41" t="s">
-        <v>1117</v>
+        <v>1114</v>
       </c>
       <c r="D184" s="41" t="s">
-        <v>1134</v>
+        <v>1131</v>
       </c>
       <c r="F184" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I184" s="41" t="s">
-        <v>1142</v>
+        <v>1139</v>
       </c>
       <c r="J184" s="96"/>
       <c r="M184" s="3" t="s">
@@ -13767,31 +13761,31 @@
     </row>
     <row r="185" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B185" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C185" s="41" t="s">
-        <v>1118</v>
+        <v>1115</v>
       </c>
       <c r="D185" s="41" t="s">
-        <v>1135</v>
+        <v>1132</v>
       </c>
       <c r="F185" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I185" s="41" t="s">
-        <v>1143</v>
+        <v>1140</v>
       </c>
       <c r="J185" s="95">
         <v>2.5</v>
       </c>
       <c r="K185" s="98" t="s">
-        <v>1257</v>
+        <v>1254</v>
       </c>
       <c r="L185" t="s">
-        <v>1238</v>
+        <v>1235</v>
       </c>
       <c r="M185" s="3" t="s">
         <v>24</v>
@@ -13814,25 +13808,25 @@
     </row>
     <row r="186" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B186" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C186" s="41" t="s">
-        <v>1119</v>
+        <v>1116</v>
       </c>
       <c r="D186" s="41" t="s">
-        <v>1136</v>
+        <v>1133</v>
       </c>
       <c r="F186" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I186" s="41" t="s">
-        <v>1144</v>
+        <v>1141</v>
       </c>
       <c r="J186" s="33" t="s">
-        <v>1194</v>
+        <v>1191</v>
       </c>
       <c r="M186" s="3" t="s">
         <v>24</v>
@@ -13855,22 +13849,22 @@
     </row>
     <row r="187" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B187" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C187" s="41" t="s">
-        <v>1120</v>
+        <v>1117</v>
       </c>
       <c r="D187" s="41" t="s">
-        <v>1138</v>
+        <v>1135</v>
       </c>
       <c r="F187" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I187" s="41" t="s">
-        <v>1145</v>
+        <v>1142</v>
       </c>
       <c r="J187" s="96"/>
       <c r="M187" s="3" t="s">
@@ -13894,22 +13888,22 @@
     </row>
     <row r="188" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B188" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C188" s="41" t="s">
-        <v>1121</v>
+        <v>1118</v>
       </c>
       <c r="D188" s="41" t="s">
-        <v>1137</v>
+        <v>1134</v>
       </c>
       <c r="F188" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I188" s="41" t="s">
-        <v>1146</v>
+        <v>1143</v>
       </c>
       <c r="J188" s="96"/>
       <c r="M188" s="3" t="s">
@@ -13933,29 +13927,29 @@
     </row>
     <row r="189" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A189" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B189" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C189" s="41" t="s">
-        <v>1122</v>
+        <v>1119</v>
       </c>
       <c r="D189" s="41" t="s">
-        <v>1130</v>
+        <v>1127</v>
       </c>
       <c r="F189" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I189" s="41" t="s">
-        <v>1147</v>
+        <v>1144</v>
       </c>
       <c r="J189" s="3"/>
       <c r="K189" s="3" t="s">
         <v>201</v>
       </c>
       <c r="L189" s="3" t="s">
-        <v>1233</v>
+        <v>1230</v>
       </c>
       <c r="M189" s="3" t="s">
         <v>24</v>
@@ -13978,22 +13972,22 @@
     </row>
     <row r="190" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A190" s="8" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B190" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C190" s="41" t="s">
-        <v>1123</v>
+        <v>1120</v>
       </c>
       <c r="D190" s="41" t="s">
-        <v>1148</v>
+        <v>1145</v>
       </c>
       <c r="F190" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I190" s="41" t="s">
-        <v>1149</v>
+        <v>1146</v>
       </c>
       <c r="J190" s="3"/>
       <c r="M190" s="3" t="s">
@@ -14040,13 +14034,13 @@
         <v>22</v>
       </c>
       <c r="J191" s="44" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="K191" s="44" t="s">
         <v>23</v>
       </c>
       <c r="L191" s="44" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M191" s="44" t="s">
         <v>24</v>
@@ -14076,7 +14070,7 @@
         <v>19</v>
       </c>
       <c r="C192" t="s">
-        <v>1099</v>
+        <v>1096</v>
       </c>
       <c r="D192" t="s">
         <v>682</v>
@@ -14085,19 +14079,19 @@
         <v>1</v>
       </c>
       <c r="G192" s="1" t="s">
-        <v>1212</v>
+        <v>1209</v>
       </c>
       <c r="I192" s="3" t="s">
-        <v>1157</v>
+        <v>1154</v>
       </c>
       <c r="J192" s="3" t="s">
-        <v>1255</v>
+        <v>1252</v>
       </c>
       <c r="K192" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L192" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M192" s="3" t="s">
         <v>24</v>
@@ -14138,16 +14132,16 @@
         <v>277</v>
       </c>
       <c r="I193" s="3" t="s">
-        <v>1156</v>
+        <v>1153</v>
       </c>
       <c r="J193" s="3" t="s">
-        <v>1252</v>
+        <v>1249</v>
       </c>
       <c r="K193" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L193" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M193" s="3" t="s">
         <v>24</v>
@@ -14176,28 +14170,28 @@
         <v>19</v>
       </c>
       <c r="C194" t="s">
-        <v>1100</v>
+        <v>1097</v>
       </c>
       <c r="D194" s="3" t="s">
-        <v>1127</v>
+        <v>1124</v>
       </c>
       <c r="F194" s="1" t="b">
         <v>0</v>
       </c>
       <c r="H194" s="1" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="I194" s="3" t="s">
-        <v>1150</v>
+        <v>1147</v>
       </c>
       <c r="J194" s="3" t="s">
-        <v>1247</v>
+        <v>1244</v>
       </c>
       <c r="K194" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L194" s="3" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="M194" s="3" t="s">
         <v>24</v>
@@ -14235,10 +14229,10 @@
         <v>0</v>
       </c>
       <c r="I195" s="3" t="s">
-        <v>1158</v>
+        <v>1155</v>
       </c>
       <c r="J195" s="3" t="s">
-        <v>1256</v>
+        <v>1253</v>
       </c>
       <c r="M195" s="3" t="s">
         <v>24</v>
@@ -14267,26 +14261,26 @@
         <v>19</v>
       </c>
       <c r="C196" t="s">
-        <v>1200</v>
+        <v>1197</v>
       </c>
       <c r="D196" s="3" t="s">
-        <v>1169</v>
+        <v>1166</v>
       </c>
       <c r="F196" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G196" s="43"/>
       <c r="I196" s="41" t="s">
-        <v>1162</v>
+        <v>1159</v>
       </c>
       <c r="J196" s="93" t="s">
-        <v>1254</v>
+        <v>1251</v>
       </c>
       <c r="K196" s="3" t="s">
-        <v>1213</v>
+        <v>1210</v>
       </c>
       <c r="L196" s="3" t="s">
-        <v>1237</v>
+        <v>1234</v>
       </c>
       <c r="M196" s="3" t="s">
         <v>24</v>
@@ -14315,20 +14309,20 @@
         <v>19</v>
       </c>
       <c r="C197" s="41" t="s">
-        <v>1159</v>
+        <v>1156</v>
       </c>
       <c r="D197" s="3" t="s">
-        <v>1164</v>
+        <v>1161</v>
       </c>
       <c r="F197" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G197" s="43"/>
       <c r="I197" s="3" t="s">
-        <v>1160</v>
+        <v>1157</v>
       </c>
       <c r="J197" s="68" t="s">
-        <v>1180</v>
+        <v>1177</v>
       </c>
       <c r="M197" s="3" t="s">
         <v>24</v>
@@ -14357,17 +14351,17 @@
         <v>19</v>
       </c>
       <c r="C198" s="41" t="s">
-        <v>1110</v>
+        <v>1107</v>
       </c>
       <c r="D198" s="41" t="s">
-        <v>1165</v>
+        <v>1162</v>
       </c>
       <c r="F198" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G198" s="43"/>
       <c r="I198" s="41" t="s">
-        <v>1151</v>
+        <v>1148</v>
       </c>
       <c r="J198" s="3">
         <v>4</v>
@@ -14376,7 +14370,7 @@
         <v>241</v>
       </c>
       <c r="L198" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M198" s="3" t="s">
         <v>24</v>
@@ -14405,17 +14399,17 @@
         <v>19</v>
       </c>
       <c r="C199" s="41" t="s">
-        <v>1111</v>
+        <v>1108</v>
       </c>
       <c r="D199" s="41" t="s">
-        <v>1166</v>
+        <v>1163</v>
       </c>
       <c r="F199" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G199" s="43"/>
       <c r="I199" s="41" t="s">
-        <v>1152</v>
+        <v>1149</v>
       </c>
       <c r="J199" s="3">
         <v>50</v>
@@ -14424,7 +14418,7 @@
         <v>241</v>
       </c>
       <c r="L199" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M199" s="3" t="s">
         <v>24</v>
@@ -14453,17 +14447,17 @@
         <v>19</v>
       </c>
       <c r="C200" s="41" t="s">
-        <v>1125</v>
+        <v>1122</v>
       </c>
       <c r="D200" s="41" t="s">
-        <v>1167</v>
+        <v>1164</v>
       </c>
       <c r="F200" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G200" s="43"/>
       <c r="I200" s="41" t="s">
-        <v>1161</v>
+        <v>1158</v>
       </c>
       <c r="J200" s="3">
         <v>90</v>
@@ -14472,7 +14466,7 @@
         <v>241</v>
       </c>
       <c r="L200" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="M200" s="3" t="s">
         <v>24</v>
@@ -14501,17 +14495,17 @@
         <v>19</v>
       </c>
       <c r="C201" s="41" t="s">
-        <v>1126</v>
+        <v>1123</v>
       </c>
       <c r="D201" s="41" t="s">
-        <v>1168</v>
+        <v>1165</v>
       </c>
       <c r="F201" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G201" s="43"/>
       <c r="I201" s="41" t="s">
-        <v>1163</v>
+        <v>1160</v>
       </c>
       <c r="J201" s="3" t="s">
         <v>53</v>
@@ -14520,7 +14514,7 @@
         <v>54</v>
       </c>
       <c r="L201" s="3" t="s">
-        <v>1225</v>
+        <v>1222</v>
       </c>
       <c r="M201" s="3" t="s">
         <v>24</v>
@@ -14734,25 +14728,25 @@
         <v>429</v>
       </c>
       <c r="AA1" s="79" t="s">
-        <v>1101</v>
+        <v>1098</v>
       </c>
       <c r="AB1" s="79" t="s">
         <v>102</v>
       </c>
       <c r="AC1" s="90" t="s">
-        <v>1109</v>
+        <v>1106</v>
       </c>
       <c r="AD1" s="90" t="s">
-        <v>1159</v>
+        <v>1156</v>
       </c>
       <c r="AE1" s="80" t="s">
-        <v>1113</v>
+        <v>1110</v>
       </c>
       <c r="AF1" s="80" t="s">
-        <v>1115</v>
+        <v>1112</v>
       </c>
       <c r="AG1" s="81" t="s">
-        <v>1119</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="2" spans="1:33" ht="16" x14ac:dyDescent="0.2">
@@ -14838,22 +14832,22 @@
         <v>728</v>
       </c>
       <c r="AB2" s="36" t="s">
-        <v>1102</v>
+        <v>1099</v>
       </c>
       <c r="AC2" s="73" t="s">
-        <v>1170</v>
+        <v>1167</v>
       </c>
       <c r="AD2" s="74" t="s">
-        <v>1176</v>
+        <v>1173</v>
       </c>
       <c r="AE2" s="73" t="s">
-        <v>1181</v>
+        <v>1178</v>
       </c>
       <c r="AF2" s="73" t="s">
-        <v>1186</v>
+        <v>1183</v>
       </c>
       <c r="AG2" s="74" t="s">
-        <v>1192</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="3" spans="1:33" ht="16" x14ac:dyDescent="0.2">
@@ -14939,22 +14933,22 @@
         <v>745</v>
       </c>
       <c r="AB3" s="36" t="s">
-        <v>1103</v>
+        <v>1100</v>
       </c>
       <c r="AC3" s="36" t="s">
-        <v>1171</v>
+        <v>1168</v>
       </c>
       <c r="AD3" s="70" t="s">
-        <v>1177</v>
+        <v>1174</v>
       </c>
       <c r="AE3" s="36" t="s">
-        <v>1182</v>
+        <v>1179</v>
       </c>
       <c r="AF3" s="36" t="s">
-        <v>1187</v>
+        <v>1184</v>
       </c>
       <c r="AG3" s="70" t="s">
-        <v>1193</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="4" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.2">
@@ -15028,22 +15022,22 @@
         <v>762</v>
       </c>
       <c r="AB4" s="36" t="s">
-        <v>1107</v>
+        <v>1104</v>
       </c>
       <c r="AC4" s="36" t="s">
-        <v>1172</v>
+        <v>1169</v>
       </c>
       <c r="AD4" s="35" t="s">
-        <v>1178</v>
+        <v>1175</v>
       </c>
       <c r="AE4" s="36" t="s">
-        <v>1183</v>
+        <v>1180</v>
       </c>
       <c r="AF4" s="36" t="s">
-        <v>1188</v>
+        <v>1185</v>
       </c>
       <c r="AG4" s="35" t="s">
-        <v>1194</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="5" spans="1:33" ht="16" x14ac:dyDescent="0.2">
@@ -15111,22 +15105,22 @@
         <v>777</v>
       </c>
       <c r="AB5" s="36" t="s">
-        <v>1104</v>
+        <v>1101</v>
       </c>
       <c r="AC5" s="36" t="s">
-        <v>1173</v>
+        <v>1170</v>
       </c>
       <c r="AD5" s="35" t="s">
-        <v>1179</v>
+        <v>1176</v>
       </c>
       <c r="AE5" s="36" t="s">
-        <v>1184</v>
+        <v>1181</v>
       </c>
       <c r="AF5" s="36" t="s">
-        <v>1189</v>
+        <v>1186</v>
       </c>
       <c r="AG5" s="35" t="s">
-        <v>1195</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="6" spans="1:33" ht="16" x14ac:dyDescent="0.2">
@@ -15184,22 +15178,22 @@
         <v>789</v>
       </c>
       <c r="AB6" s="36" t="s">
-        <v>1105</v>
+        <v>1102</v>
       </c>
       <c r="AC6" s="36" t="s">
-        <v>1174</v>
+        <v>1171</v>
       </c>
       <c r="AD6" s="36" t="s">
-        <v>1180</v>
+        <v>1177</v>
       </c>
       <c r="AE6" s="36" t="s">
-        <v>1185</v>
+        <v>1182</v>
       </c>
       <c r="AF6" s="36" t="s">
-        <v>1190</v>
+        <v>1187</v>
       </c>
       <c r="AG6" s="35" t="s">
-        <v>1196</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="7" spans="1:33" ht="16" x14ac:dyDescent="0.2">
@@ -15251,18 +15245,18 @@
         <v>105</v>
       </c>
       <c r="AB7" s="36" t="s">
-        <v>1106</v>
+        <v>1103</v>
       </c>
       <c r="AC7" s="36" t="s">
-        <v>1175</v>
+        <v>1172</v>
       </c>
       <c r="AD7" s="36"/>
       <c r="AE7" s="36"/>
       <c r="AF7" s="36" t="s">
-        <v>1191</v>
+        <v>1188</v>
       </c>
       <c r="AG7" s="35" t="s">
-        <v>1197</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="8" spans="1:33" ht="16" x14ac:dyDescent="0.2">
@@ -26218,10 +26212,10 @@
         <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>1214</v>
+        <v>1211</v>
       </c>
       <c r="C2" t="s">
-        <v>1215</v>
+        <v>1212</v>
       </c>
       <c r="D2" t="s">
         <v>941</v>
@@ -26235,10 +26229,10 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>1216</v>
+        <v>1213</v>
       </c>
       <c r="C3" t="s">
-        <v>1217</v>
+        <v>1214</v>
       </c>
       <c r="D3" t="s">
         <v>35</v>
@@ -26252,10 +26246,10 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>1218</v>
+        <v>1215</v>
       </c>
       <c r="C4" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="D4" t="s">
         <v>242</v>
@@ -26269,10 +26263,10 @@
         <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>1220</v>
+        <v>1217</v>
       </c>
       <c r="C5" t="s">
-        <v>1221</v>
+        <v>1218</v>
       </c>
       <c r="D5" t="s">
         <v>89</v>
@@ -26308,10 +26302,10 @@
         <v>939</v>
       </c>
       <c r="C1" s="16" t="s">
+        <v>943</v>
+      </c>
+      <c r="D1" s="16" t="s">
         <v>944</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>945</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -26319,7 +26313,7 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="C2" t="s">
         <v>18</v>
@@ -26333,7 +26327,7 @@
         <v>106</v>
       </c>
       <c r="B3" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -26349,7 +26343,7 @@
         <v>170</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -26357,7 +26351,7 @@
         <v>226</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -26365,7 +26359,7 @@
         <v>277</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -26373,7 +26367,7 @@
         <v>435</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -26381,7 +26375,7 @@
         <v>514</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -26389,7 +26383,7 @@
         <v>530</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -26397,7 +26391,7 @@
         <v>631</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -26405,7 +26399,7 @@
         <v>642</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -26413,18 +26407,18 @@
         <v>519</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>955</v>
+      </c>
+      <c r="C13" t="s">
         <v>956</v>
-      </c>
-      <c r="C13" t="s">
-        <v>957</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="45" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1198</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="17" thickTop="1" x14ac:dyDescent="0.2">
@@ -26457,7 +26451,7 @@
         <v>938</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -26467,12 +26461,12 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
   </sheetData>
@@ -26500,10 +26494,10 @@
         <v>9</v>
       </c>
       <c r="B1" s="20" t="s">
+        <v>960</v>
+      </c>
+      <c r="C1" s="20" t="s">
         <v>961</v>
-      </c>
-      <c r="C1" s="20" t="s">
-        <v>962</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -26511,21 +26505,21 @@
         <v>23</v>
       </c>
       <c r="B2" s="21" t="s">
+        <v>962</v>
+      </c>
+      <c r="C2" s="22" t="s">
         <v>963</v>
-      </c>
-      <c r="C2" s="22" t="s">
-        <v>964</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="21" t="s">
+        <v>964</v>
+      </c>
+      <c r="B3" s="21" t="s">
         <v>965</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="C3" s="22" t="s">
         <v>966</v>
-      </c>
-      <c r="C3" s="22" t="s">
-        <v>967</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -26533,43 +26527,43 @@
         <v>129</v>
       </c>
       <c r="B4" s="21" t="s">
+        <v>967</v>
+      </c>
+      <c r="C4" s="22" t="s">
         <v>968</v>
-      </c>
-      <c r="C4" s="22" t="s">
-        <v>969</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="21" t="s">
+        <v>969</v>
+      </c>
+      <c r="B5" s="21" t="s">
         <v>970</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="C5" s="22" t="s">
         <v>971</v>
-      </c>
-      <c r="C5" s="22" t="s">
-        <v>972</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="21" t="s">
+        <v>972</v>
+      </c>
+      <c r="B6" s="21" t="s">
         <v>973</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="C6" s="22" t="s">
         <v>974</v>
-      </c>
-      <c r="C6" s="22" t="s">
-        <v>975</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="21" t="s">
+        <v>975</v>
+      </c>
+      <c r="B7" s="21" t="s">
         <v>976</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="C7" s="22" t="s">
         <v>977</v>
-      </c>
-      <c r="C7" s="22" t="s">
-        <v>978</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -26577,7 +26571,7 @@
         <v>80</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="C8" s="22"/>
     </row>
@@ -26586,16 +26580,16 @@
         <v>98</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="C9" s="22"/>
     </row>
     <row r="10" spans="1:3" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="21" t="s">
+        <v>980</v>
+      </c>
+      <c r="B10" s="21" t="s">
         <v>981</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>982</v>
       </c>
       <c r="C10" s="22"/>
     </row>
@@ -26604,63 +26598,63 @@
         <v>241</v>
       </c>
       <c r="B11" s="21" t="s">
+        <v>982</v>
+      </c>
+      <c r="C11" s="22" t="s">
         <v>983</v>
-      </c>
-      <c r="C11" s="22" t="s">
-        <v>984</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="21" t="s">
+        <v>984</v>
+      </c>
+      <c r="B12" s="21" t="s">
         <v>985</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>986</v>
       </c>
       <c r="C12" s="22"/>
     </row>
     <row r="13" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="21" t="s">
+        <v>986</v>
+      </c>
+      <c r="B13" s="21" t="s">
         <v>987</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="C13" s="22" t="s">
         <v>988</v>
-      </c>
-      <c r="C13" s="22" t="s">
-        <v>989</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="21" t="s">
+        <v>989</v>
+      </c>
+      <c r="B14" s="21" t="s">
         <v>990</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="C14" s="22" t="s">
         <v>991</v>
-      </c>
-      <c r="C14" s="22" t="s">
-        <v>992</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="21" t="s">
+        <v>992</v>
+      </c>
+      <c r="B15" s="21" t="s">
         <v>993</v>
       </c>
-      <c r="B15" s="21" t="s">
+      <c r="C15" s="22" t="s">
         <v>994</v>
-      </c>
-      <c r="C15" s="22" t="s">
-        <v>995</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="21" t="s">
+        <v>995</v>
+      </c>
+      <c r="B16" s="21" t="s">
         <v>996</v>
       </c>
-      <c r="B16" s="21" t="s">
+      <c r="C16" s="22" t="s">
         <v>997</v>
-      </c>
-      <c r="C16" s="22" t="s">
-        <v>998</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -26668,21 +26662,21 @@
         <v>676</v>
       </c>
       <c r="B17" s="21" t="s">
+        <v>998</v>
+      </c>
+      <c r="C17" s="22" t="s">
         <v>999</v>
-      </c>
-      <c r="C17" s="22" t="s">
-        <v>1000</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="21" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B18" s="21" t="s">
         <v>1001</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="C18" s="22" t="s">
         <v>1002</v>
-      </c>
-      <c r="C18" s="22" t="s">
-        <v>1003</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -26690,25 +26684,25 @@
         <v>390</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="C19" s="22"/>
     </row>
     <row r="20" spans="1:3" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="17" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B20" s="21" t="s">
         <v>1005</v>
-      </c>
-      <c r="B20" s="21" t="s">
-        <v>1006</v>
       </c>
       <c r="C20" s="22"/>
     </row>
     <row r="21" spans="1:3" ht="41.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="21" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B21" s="21" t="s">
         <v>1007</v>
-      </c>
-      <c r="B21" s="21" t="s">
-        <v>1008</v>
       </c>
       <c r="C21" s="22"/>
     </row>
@@ -26717,41 +26711,41 @@
         <v>379</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="C22" s="22"/>
     </row>
     <row r="23" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="21" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B23" s="21" t="s">
         <v>1010</v>
       </c>
-      <c r="B23" s="21" t="s">
+      <c r="C23" s="22" t="s">
         <v>1011</v>
-      </c>
-      <c r="C23" s="22" t="s">
-        <v>1012</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="21" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B24" s="21" t="s">
         <v>1013</v>
       </c>
-      <c r="B24" s="21" t="s">
+      <c r="C24" s="22" t="s">
         <v>1014</v>
-      </c>
-      <c r="C24" s="22" t="s">
-        <v>1015</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="41.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="21" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B25" s="21" t="s">
         <v>1016</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="C25" s="22" t="s">
         <v>1017</v>
-      </c>
-      <c r="C25" s="22" t="s">
-        <v>1018</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -26759,10 +26753,10 @@
         <v>201</v>
       </c>
       <c r="B26" s="21" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C26" s="22" t="s">
         <v>1019</v>
-      </c>
-      <c r="C26" s="22" t="s">
-        <v>1020</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -26770,10 +26764,10 @@
         <v>400</v>
       </c>
       <c r="B27" s="21" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C27" s="22" t="s">
         <v>1021</v>
-      </c>
-      <c r="C27" s="22" t="s">
-        <v>1022</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -26781,10 +26775,10 @@
         <v>54</v>
       </c>
       <c r="B28" s="21" t="s">
+        <v>1022</v>
+      </c>
+      <c r="C28" s="22" t="s">
         <v>1023</v>
-      </c>
-      <c r="C28" s="22" t="s">
-        <v>1024</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -26792,10 +26786,10 @@
         <v>614</v>
       </c>
       <c r="B29" s="21" t="s">
+        <v>1024</v>
+      </c>
+      <c r="C29" s="22" t="s">
         <v>1025</v>
-      </c>
-      <c r="C29" s="22" t="s">
-        <v>1026</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -26803,43 +26797,43 @@
         <v>677</v>
       </c>
       <c r="B30" s="21" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C30" s="22" t="s">
         <v>1027</v>
-      </c>
-      <c r="C30" s="22" t="s">
-        <v>1028</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="21" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B31" s="21" t="s">
         <v>1029</v>
       </c>
-      <c r="B31" s="21" t="s">
+      <c r="C31" s="22" t="s">
         <v>1030</v>
-      </c>
-      <c r="C31" s="22" t="s">
-        <v>1031</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="17" t="s">
+        <v>1031</v>
+      </c>
+      <c r="B32" s="21" t="s">
         <v>1032</v>
       </c>
-      <c r="B32" s="21" t="s">
+      <c r="C32" s="22" t="s">
         <v>1033</v>
-      </c>
-      <c r="C32" s="22" t="s">
-        <v>1034</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="21" t="s">
+        <v>1034</v>
+      </c>
+      <c r="B33" s="21" t="s">
         <v>1035</v>
       </c>
-      <c r="B33" s="21" t="s">
+      <c r="C33" s="22" t="s">
         <v>1036</v>
-      </c>
-      <c r="C33" s="22" t="s">
-        <v>1037</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.2">
@@ -26847,21 +26841,21 @@
         <v>111</v>
       </c>
       <c r="B34" s="26" t="s">
+        <v>1037</v>
+      </c>
+      <c r="C34" s="27" t="s">
         <v>1038</v>
-      </c>
-      <c r="C34" s="27" t="s">
-        <v>1039</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="26" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B35" s="26" t="s">
         <v>1040</v>
       </c>
-      <c r="B35" s="26" t="s">
+      <c r="C35" s="27" t="s">
         <v>1041</v>
-      </c>
-      <c r="C35" s="27" t="s">
-        <v>1042</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -26869,7 +26863,7 @@
         <v>679</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="C36" s="27"/>
     </row>
@@ -26878,7 +26872,7 @@
         <v>87</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="C37" s="22"/>
     </row>
@@ -26887,7 +26881,7 @@
         <v>117</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="C38" s="27"/>
     </row>
@@ -26896,7 +26890,7 @@
         <v>123</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="C39" s="22"/>
     </row>
@@ -26905,7 +26899,7 @@
         <v>135</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="C40" s="22"/>
     </row>
@@ -26914,52 +26908,52 @@
         <v>146</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="C41" s="22"/>
     </row>
     <row r="42" spans="1:3" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="26" t="s">
+        <v>1048</v>
+      </c>
+      <c r="B42" s="26" t="s">
         <v>1049</v>
-      </c>
-      <c r="B42" s="26" t="s">
-        <v>1050</v>
       </c>
       <c r="C42" s="27"/>
     </row>
     <row r="43" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="21" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B43" s="21" t="s">
         <v>1051</v>
-      </c>
-      <c r="B43" s="21" t="s">
-        <v>1052</v>
       </c>
       <c r="C43" s="22"/>
     </row>
     <row r="44" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="21" t="s">
+        <v>1052</v>
+      </c>
+      <c r="B44" s="21" t="s">
         <v>1053</v>
-      </c>
-      <c r="B44" s="21" t="s">
-        <v>1054</v>
       </c>
       <c r="C44" s="22"/>
     </row>
     <row r="45" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="21" t="s">
+        <v>1054</v>
+      </c>
+      <c r="B45" s="21" t="s">
         <v>1055</v>
-      </c>
-      <c r="B45" s="21" t="s">
-        <v>1056</v>
       </c>
       <c r="C45" s="22"/>
     </row>
     <row r="46" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="21" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B46" s="21" t="s">
         <v>1057</v>
-      </c>
-      <c r="B46" s="21" t="s">
-        <v>1058</v>
       </c>
       <c r="C46" s="22"/>
     </row>
@@ -26968,16 +26962,16 @@
         <v>225</v>
       </c>
       <c r="B47" s="26" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="C47" s="27"/>
     </row>
     <row r="48" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="21" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B48" s="21" t="s">
         <v>1060</v>
-      </c>
-      <c r="B48" s="21" t="s">
-        <v>1061</v>
       </c>
       <c r="C48" s="22"/>
     </row>
@@ -26986,61 +26980,61 @@
         <v>680</v>
       </c>
       <c r="B49" s="21" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="C49" s="22"/>
     </row>
     <row r="50" spans="1:3" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="26" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B50" s="26" t="s">
         <v>1063</v>
-      </c>
-      <c r="B50" s="26" t="s">
-        <v>1064</v>
       </c>
       <c r="C50" s="27"/>
     </row>
     <row r="51" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="26" t="s">
+        <v>1064</v>
+      </c>
+      <c r="B51" s="26" t="s">
         <v>1065</v>
-      </c>
-      <c r="B51" s="26" t="s">
-        <v>1066</v>
       </c>
       <c r="C51" s="27"/>
     </row>
     <row r="52" spans="1:3" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="21" t="s">
+        <v>1066</v>
+      </c>
+      <c r="B52" s="21" t="s">
         <v>1067</v>
-      </c>
-      <c r="B52" s="21" t="s">
-        <v>1068</v>
       </c>
       <c r="C52" s="22"/>
     </row>
     <row r="53" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="26" t="s">
+        <v>1068</v>
+      </c>
+      <c r="B53" s="26" t="s">
         <v>1069</v>
-      </c>
-      <c r="B53" s="26" t="s">
-        <v>1070</v>
       </c>
       <c r="C53" s="27"/>
     </row>
     <row r="54" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="21" t="s">
+        <v>1070</v>
+      </c>
+      <c r="B54" s="21" t="s">
         <v>1071</v>
-      </c>
-      <c r="B54" s="21" t="s">
-        <v>1072</v>
       </c>
       <c r="C54" s="22"/>
     </row>
     <row r="55" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="26" t="s">
+        <v>1072</v>
+      </c>
+      <c r="B55" s="26" t="s">
         <v>1073</v>
-      </c>
-      <c r="B55" s="26" t="s">
-        <v>1074</v>
       </c>
       <c r="C55" s="27"/>
     </row>
@@ -27049,25 +27043,25 @@
         <v>217</v>
       </c>
       <c r="B56" s="26" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="C56" s="27"/>
     </row>
     <row r="57" spans="1:3" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="26" t="s">
+        <v>1075</v>
+      </c>
+      <c r="B57" s="26" t="s">
         <v>1076</v>
-      </c>
-      <c r="B57" s="26" t="s">
-        <v>1077</v>
       </c>
       <c r="C57" s="27"/>
     </row>
     <row r="58" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="26" t="s">
+        <v>1077</v>
+      </c>
+      <c r="B58" s="26" t="s">
         <v>1078</v>
-      </c>
-      <c r="B58" s="26" t="s">
-        <v>1079</v>
       </c>
       <c r="C58" s="27"/>
     </row>
@@ -27076,34 +27070,34 @@
         <v>162</v>
       </c>
       <c r="B59" s="49" t="s">
-        <v>1098</v>
+        <v>1095</v>
       </c>
       <c r="C59" s="50"/>
     </row>
     <row r="60" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" s="49" t="s">
-        <v>1201</v>
+        <v>1198</v>
       </c>
       <c r="B60" s="49" t="s">
-        <v>1202</v>
+        <v>1199</v>
       </c>
       <c r="C60" s="50"/>
     </row>
     <row r="61" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="49" t="s">
+        <v>1256</v>
+      </c>
+      <c r="B61" s="49" t="s">
         <v>1259</v>
-      </c>
-      <c r="B61" s="49" t="s">
-        <v>1262</v>
       </c>
       <c r="C61" s="50"/>
     </row>
     <row r="62" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="49" t="s">
-        <v>1213</v>
+        <v>1210</v>
       </c>
       <c r="B62" s="49" t="s">
-        <v>1263</v>
+        <v>1260</v>
       </c>
       <c r="C62" s="50"/>
     </row>
@@ -27138,7 +27132,7 @@
         <v>941</v>
       </c>
       <c r="B2" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -27146,7 +27140,7 @@
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -27154,7 +27148,7 @@
         <v>242</v>
       </c>
       <c r="B4" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -27162,7 +27156,7 @@
         <v>89</v>
       </c>
       <c r="B5" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
   </sheetData>
@@ -27175,7 +27169,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -27195,15 +27189,7 @@
         <v>942</v>
       </c>
       <c r="B2" t="s">
-        <v>1084</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>943</v>
-      </c>
-      <c r="B3" t="s">
-        <v>1085</v>
+        <v>1264</v>
       </c>
     </row>
   </sheetData>
@@ -27231,7 +27217,7 @@
         <v>4</v>
       </c>
       <c r="B1" s="82" t="s">
-        <v>1086</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -27239,7 +27225,7 @@
         <v>159</v>
       </c>
       <c r="B2" s="36" t="s">
-        <v>1087</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -27247,31 +27233,31 @@
         <v>152</v>
       </c>
       <c r="B3" s="35" t="s">
-        <v>1088</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="68" t="s">
-        <v>1089</v>
+        <v>1086</v>
       </c>
       <c r="B4" s="36" t="s">
-        <v>1090</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="68" t="s">
-        <v>1091</v>
+        <v>1088</v>
       </c>
       <c r="B5" s="36" t="s">
-        <v>1092</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="83" t="s">
-        <v>1093</v>
+        <v>1090</v>
       </c>
       <c r="B6" s="83" t="s">
-        <v>1093</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -27284,10 +27270,10 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="68" t="s">
-        <v>1094</v>
+        <v>1091</v>
       </c>
       <c r="B8" s="68" t="s">
-        <v>1094</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -27332,26 +27318,26 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="68" t="s">
-        <v>1095</v>
+        <v>1092</v>
       </c>
       <c r="B14" s="68" t="s">
-        <v>1095</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="36" t="s">
-        <v>1096</v>
+        <v>1093</v>
       </c>
       <c r="B15" s="36" t="s">
-        <v>1096</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="68" t="s">
-        <v>1097</v>
+        <v>1094</v>
       </c>
       <c r="B16" s="68" t="s">
-        <v>1097</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
CD-182: Added missing enums for 'library_strategy', 'library_selection' and 'library_source' fields in Single-cell schema
- Added 'NOMe-Seq' option to 'library_strategy' field
- Added 'cDNA_oligo_dT'
'cDNA_randomPriming',
'Dnase', 'Mnase', 'Inverse rRNA' and 'PolyA' options to 'library_selection' field
- Added 'GENOMIC SINGLE CELL' and
'TRANSCRIPTOMIC SINGLE CELL' options to 'library_source' field
</commit_message>
<xml_diff>
--- a/single_cell/singlecell_schema_main_v0.4.xlsx
+++ b/single_cell/singlecell_schema_main_v0.4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/providen/Documents/EI/Projects/COPO-schemas/single_cell/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{118AE7D9-7D3B-BE48-BB38-532C475A47CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82992FDF-4828-5E4A-9195-C924823E24B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31760" yWindow="340" windowWidth="30240" windowHeight="18080" activeTab="7" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
+    <workbookView xWindow="30240" yWindow="-2660" windowWidth="38400" windowHeight="21600" activeTab="1" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3121" uniqueCount="1265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3128" uniqueCount="1272">
   <si>
     <t>component_name</t>
   </si>
@@ -2566,16 +2566,10 @@
     <t>WGS</t>
   </si>
   <si>
-    <t>MNase</t>
-  </si>
-  <si>
     <t>Illumina HiSeq 1000</t>
   </si>
   <si>
     <t>WCS</t>
-  </si>
-  <si>
-    <t>DNase</t>
   </si>
   <si>
     <t>Illumina HiSeq 1500</t>
@@ -4008,6 +4002,33 @@
   </si>
   <si>
     <t>Single-cell Ribonucleic Acid Sequencing (scRNA-Seq)</t>
+  </si>
+  <si>
+    <t>GENOMIC SINGLE CELL</t>
+  </si>
+  <si>
+    <t>TRANSCRIPTOMIC SINGLE CELL</t>
+  </si>
+  <si>
+    <t>cDNA_randomPriming</t>
+  </si>
+  <si>
+    <t>PolyA</t>
+  </si>
+  <si>
+    <t>cDNA_oligo_dT</t>
+  </si>
+  <si>
+    <t>Inverse rRNA</t>
+  </si>
+  <si>
+    <t>Mnase</t>
+  </si>
+  <si>
+    <t>Dnase</t>
+  </si>
+  <si>
+    <t>NOMe-Seq</t>
   </si>
 </sst>
 </file>
@@ -5415,7 +5436,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>1202</v>
+        <v>1200</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>6</v>
@@ -5474,13 +5495,13 @@
         <v>22</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>24</v>
@@ -5708,7 +5729,7 @@
         <v>54</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>1222</v>
+        <v>1220</v>
       </c>
       <c r="M7" s="3" t="s">
         <v>24</v>
@@ -5881,7 +5902,7 @@
         <v>23</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M11" s="3" t="s">
         <v>24</v>
@@ -5922,10 +5943,10 @@
         <v>79</v>
       </c>
       <c r="K12" s="3" t="s">
+        <v>1254</v>
+      </c>
+      <c r="L12" s="3" t="s">
         <v>1256</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>1258</v>
       </c>
       <c r="M12" s="3" t="s">
         <v>81</v>
@@ -5969,7 +5990,7 @@
         <v>87</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>1223</v>
+        <v>1221</v>
       </c>
       <c r="M13" s="3" t="s">
         <v>24</v>
@@ -6051,7 +6072,7 @@
         <v>98</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>1224</v>
+        <v>1222</v>
       </c>
       <c r="M15" s="3" t="s">
         <v>24</v>
@@ -6128,7 +6149,7 @@
         <v>104</v>
       </c>
       <c r="J17" t="s">
-        <v>1103</v>
+        <v>1101</v>
       </c>
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
@@ -6177,13 +6198,13 @@
         <v>22</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M18" s="2" t="s">
         <v>24</v>
@@ -6231,7 +6252,7 @@
         <v>111</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>1225</v>
+        <v>1223</v>
       </c>
       <c r="M19" s="3" t="s">
         <v>24</v>
@@ -6279,7 +6300,7 @@
         <v>117</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>1223</v>
+        <v>1221</v>
       </c>
       <c r="M20" s="3" t="s">
         <v>24</v>
@@ -6329,7 +6350,7 @@
         <v>123</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>1223</v>
+        <v>1221</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>24</v>
@@ -6379,7 +6400,7 @@
         <v>129</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="M22" s="3" t="s">
         <v>24</v>
@@ -6429,7 +6450,7 @@
         <v>135</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>1223</v>
+        <v>1221</v>
       </c>
       <c r="M23" s="3" t="s">
         <v>24</v>
@@ -6525,7 +6546,7 @@
         <v>146</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>1223</v>
+        <v>1221</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>24</v>
@@ -6574,13 +6595,13 @@
         <v>149</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="K26" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M26" s="2" t="s">
         <v>24</v>
@@ -6619,10 +6640,10 @@
         <v>1</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>1263</v>
+        <v>1261</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>1248</v>
+        <v>1246</v>
       </c>
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
@@ -6651,7 +6672,7 @@
         <v>148</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>152</v>
@@ -6675,7 +6696,7 @@
         <v>135</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>1227</v>
+        <v>1225</v>
       </c>
       <c r="M28" s="3" t="s">
         <v>24</v>
@@ -6704,7 +6725,7 @@
         <v>148</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>159</v>
@@ -6728,7 +6749,7 @@
         <v>162</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M29" s="3" t="s">
         <v>24</v>
@@ -6757,7 +6778,7 @@
         <v>148</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>164</v>
@@ -6826,13 +6847,13 @@
         <v>22</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="K31" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M31" s="2" t="s">
         <v>24</v>
@@ -6871,19 +6892,19 @@
         <v>1</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>1203</v>
+        <v>1201</v>
       </c>
       <c r="I32" s="3" t="s">
         <v>173</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>1245</v>
+        <v>1243</v>
       </c>
       <c r="K32" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M32" s="3" t="s">
         <v>24</v>
@@ -7137,7 +7158,7 @@
         <v>193</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>1257</v>
+        <v>1255</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>194</v>
@@ -7155,7 +7176,7 @@
         <v>87</v>
       </c>
       <c r="L38" s="3" t="s">
-        <v>1223</v>
+        <v>1221</v>
       </c>
       <c r="M38" s="3" t="s">
         <v>24</v>
@@ -7206,7 +7227,7 @@
         <v>201</v>
       </c>
       <c r="L39" s="3" t="s">
-        <v>1230</v>
+        <v>1228</v>
       </c>
       <c r="M39" s="3" t="s">
         <v>24</v>
@@ -7374,22 +7395,22 @@
         <v>216</v>
       </c>
       <c r="J43" s="17" t="s">
-        <v>1220</v>
+        <v>1218</v>
       </c>
       <c r="K43" s="3" t="s">
         <v>217</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>1223</v>
+        <v>1221</v>
       </c>
       <c r="M43" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N43" s="92" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="O43" s="13" t="s">
-        <v>1201</v>
+        <v>1199</v>
       </c>
       <c r="P43" s="31"/>
       <c r="Q43" s="56"/>
@@ -7465,7 +7486,7 @@
         <v>225</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>1223</v>
+        <v>1221</v>
       </c>
       <c r="M45" s="3" t="s">
         <v>24</v>
@@ -7506,13 +7527,13 @@
         <v>22</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="K46" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>1229</v>
+        <v>1227</v>
       </c>
       <c r="M46" s="2" t="s">
         <v>24</v>
@@ -7551,19 +7572,19 @@
         <v>1</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>1204</v>
+        <v>1202</v>
       </c>
       <c r="I47" s="3" t="s">
         <v>229</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
       <c r="K47" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L47" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M47" s="3" t="s">
         <v>24</v>
@@ -7605,10 +7626,10 @@
         <v>148</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>1261</v>
+        <v>1259</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>1248</v>
+        <v>1246</v>
       </c>
       <c r="K48" s="3"/>
       <c r="L48" s="3"/>
@@ -7655,13 +7676,13 @@
         <v>173</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>1245</v>
+        <v>1243</v>
       </c>
       <c r="K49" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L49" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M49" s="3" t="s">
         <v>24</v>
@@ -7751,7 +7772,7 @@
         <v>201</v>
       </c>
       <c r="L51" t="s">
-        <v>1230</v>
+        <v>1228</v>
       </c>
       <c r="M51" s="3" t="s">
         <v>24</v>
@@ -7796,7 +7817,7 @@
         <v>241</v>
       </c>
       <c r="L52" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M52" s="3" t="s">
         <v>24</v>
@@ -8151,7 +8172,7 @@
         <v>241</v>
       </c>
       <c r="L60" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M60" s="3" t="s">
         <v>24</v>
@@ -8243,7 +8264,7 @@
         <v>225</v>
       </c>
       <c r="L62" s="3" t="s">
-        <v>1223</v>
+        <v>1221</v>
       </c>
       <c r="M62" s="3" t="s">
         <v>24</v>
@@ -8284,13 +8305,13 @@
         <v>22</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="K63" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M63" s="2" t="s">
         <v>24</v>
@@ -8329,19 +8350,19 @@
         <v>1</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>1205</v>
+        <v>1203</v>
       </c>
       <c r="I64" s="3" t="s">
         <v>280</v>
       </c>
       <c r="J64" s="3" t="s">
-        <v>1249</v>
+        <v>1247</v>
       </c>
       <c r="K64" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L64" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M64" s="3" t="s">
         <v>24</v>
@@ -8386,13 +8407,13 @@
         <v>281</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
       <c r="K65" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L65" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M65" s="3" t="s">
         <v>24</v>
@@ -8434,10 +8455,10 @@
         <v>148</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>1262</v>
+        <v>1260</v>
       </c>
       <c r="J66" s="3" t="s">
-        <v>1248</v>
+        <v>1246</v>
       </c>
       <c r="K66" s="3"/>
       <c r="L66" s="3"/>
@@ -8504,7 +8525,7 @@
         <v>277</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C68" s="3" t="s">
         <v>287</v>
@@ -8525,7 +8546,7 @@
         <v>241</v>
       </c>
       <c r="L68" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M68" s="3" t="s">
         <v>24</v>
@@ -8622,7 +8643,7 @@
         <v>241</v>
       </c>
       <c r="L70" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M70" s="3" t="s">
         <v>24</v>
@@ -8670,7 +8691,7 @@
         <v>241</v>
       </c>
       <c r="L71" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M71" s="3" t="s">
         <v>24</v>
@@ -9328,13 +9349,13 @@
         <v>362</v>
       </c>
       <c r="J86" s="3" t="s">
-        <v>1255</v>
+        <v>1253</v>
       </c>
       <c r="K86" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L86" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M86" s="3" t="s">
         <v>24</v>
@@ -9426,7 +9447,7 @@
         <v>241</v>
       </c>
       <c r="L88" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M88" s="3" t="s">
         <v>24</v>
@@ -9521,7 +9542,7 @@
         <v>379</v>
       </c>
       <c r="L90" t="s">
-        <v>1233</v>
+        <v>1231</v>
       </c>
       <c r="M90" s="3" t="s">
         <v>24</v>
@@ -9565,7 +9586,7 @@
         <v>379</v>
       </c>
       <c r="L91" t="s">
-        <v>1233</v>
+        <v>1231</v>
       </c>
       <c r="M91" s="3" t="s">
         <v>24</v>
@@ -9609,7 +9630,7 @@
         <v>390</v>
       </c>
       <c r="L92" s="3" t="s">
-        <v>1236</v>
+        <v>1234</v>
       </c>
       <c r="M92" s="3" t="s">
         <v>24</v>
@@ -9693,7 +9714,7 @@
         <v>400</v>
       </c>
       <c r="L94" s="3" t="s">
-        <v>1232</v>
+        <v>1230</v>
       </c>
       <c r="M94" s="3" t="s">
         <v>24</v>
@@ -9851,13 +9872,13 @@
         <v>419</v>
       </c>
       <c r="J98" s="91" t="s">
-        <v>1219</v>
+        <v>1217</v>
       </c>
       <c r="K98" s="3" t="s">
         <v>54</v>
       </c>
       <c r="L98" s="3" t="s">
-        <v>1222</v>
+        <v>1220</v>
       </c>
       <c r="M98" s="3" t="s">
         <v>24</v>
@@ -9896,7 +9917,7 @@
         <v>201</v>
       </c>
       <c r="L99" s="3" t="s">
-        <v>1230</v>
+        <v>1228</v>
       </c>
       <c r="M99" s="3" t="s">
         <v>24</v>
@@ -10119,13 +10140,13 @@
         <v>22</v>
       </c>
       <c r="J104" s="2" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="K104" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L104" s="2" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M104" s="2" t="s">
         <v>24</v>
@@ -10152,7 +10173,7 @@
         <v>435</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C105" s="3" t="s">
         <v>436</v>
@@ -10164,19 +10185,19 @@
         <v>1</v>
       </c>
       <c r="G105" s="1" t="s">
-        <v>1206</v>
+        <v>1204</v>
       </c>
       <c r="I105" s="3" t="s">
         <v>438</v>
       </c>
       <c r="J105" s="3" t="s">
-        <v>1250</v>
+        <v>1248</v>
       </c>
       <c r="K105" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L105" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M105" s="3" t="s">
         <v>24</v>
@@ -10205,7 +10226,7 @@
         <v>435</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C106" s="3" t="s">
         <v>440</v>
@@ -10251,7 +10272,7 @@
         <v>435</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C107" s="3" t="s">
         <v>445</v>
@@ -10414,7 +10435,7 @@
         <v>241</v>
       </c>
       <c r="L110" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M110" s="3" t="s">
         <v>24</v>
@@ -10462,7 +10483,7 @@
         <v>241</v>
       </c>
       <c r="L111" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M111" s="3" t="s">
         <v>24</v>
@@ -10489,7 +10510,7 @@
         <v>435</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C112" s="3" t="s">
         <v>467</v>
@@ -10535,7 +10556,7 @@
         <v>435</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C113" s="3" t="s">
         <v>472</v>
@@ -10556,7 +10577,7 @@
         <v>241</v>
       </c>
       <c r="L113" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M113" s="3" t="s">
         <v>24</v>
@@ -10585,7 +10606,7 @@
         <v>435</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C114" s="3" t="s">
         <v>476</v>
@@ -10606,7 +10627,7 @@
         <v>241</v>
       </c>
       <c r="L114" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M114" s="3" t="s">
         <v>24</v>
@@ -10635,7 +10656,7 @@
         <v>435</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C115" s="3" t="s">
         <v>479</v>
@@ -10681,7 +10702,7 @@
         <v>435</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C116" s="3" t="s">
         <v>484</v>
@@ -10702,7 +10723,7 @@
         <v>241</v>
       </c>
       <c r="L116" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M116" s="3" t="s">
         <v>24</v>
@@ -10731,7 +10752,7 @@
         <v>435</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C117" s="3" t="s">
         <v>488</v>
@@ -10752,7 +10773,7 @@
         <v>241</v>
       </c>
       <c r="L117" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M117" s="3" t="s">
         <v>24</v>
@@ -10802,7 +10823,7 @@
         <v>241</v>
       </c>
       <c r="L118" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M118" s="3" t="s">
         <v>24</v>
@@ -10886,7 +10907,7 @@
         <v>241</v>
       </c>
       <c r="L120" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M120" s="3" t="s">
         <v>24</v>
@@ -10970,7 +10991,7 @@
         <v>241</v>
       </c>
       <c r="L122" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M122" s="3" t="s">
         <v>24</v>
@@ -11013,13 +11034,13 @@
         <v>22</v>
       </c>
       <c r="J123" s="2" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="K123" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L123" s="2" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M123" s="2" t="s">
         <v>24</v>
@@ -11242,13 +11263,13 @@
         <v>22</v>
       </c>
       <c r="J128" s="2" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="K128" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L128" s="2" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M128" s="2" t="s">
         <v>24</v>
@@ -11952,7 +11973,7 @@
         <v>241</v>
       </c>
       <c r="L144" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M144" s="3" t="s">
         <v>24</v>
@@ -12116,7 +12137,7 @@
         <v>614</v>
       </c>
       <c r="L148" s="3" t="s">
-        <v>1231</v>
+        <v>1229</v>
       </c>
       <c r="M148" s="3" t="s">
         <v>24</v>
@@ -12200,7 +12221,7 @@
         <v>614</v>
       </c>
       <c r="L150" s="3" t="s">
-        <v>1231</v>
+        <v>1229</v>
       </c>
       <c r="M150" s="3" t="s">
         <v>24</v>
@@ -12283,13 +12304,13 @@
         <v>22</v>
       </c>
       <c r="J152" s="2" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="K152" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L152" s="2" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M152" s="2" t="s">
         <v>24</v>
@@ -12560,7 +12581,7 @@
         <v>23</v>
       </c>
       <c r="L158" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M158" s="3" t="s">
         <v>24</v>
@@ -12827,13 +12848,13 @@
         <v>22</v>
       </c>
       <c r="J164" s="2" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="K164" s="2" t="s">
         <v>23</v>
       </c>
       <c r="L164" s="2" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M164" s="2" t="s">
         <v>24</v>
@@ -12872,19 +12893,19 @@
         <v>1</v>
       </c>
       <c r="G165" s="1" t="s">
-        <v>1207</v>
+        <v>1205</v>
       </c>
       <c r="I165" s="3" t="s">
         <v>683</v>
       </c>
       <c r="J165" s="3" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="K165" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L165" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M165" s="3" t="s">
         <v>24</v>
@@ -12929,13 +12950,13 @@
         <v>280</v>
       </c>
       <c r="J166" s="3" t="s">
-        <v>1249</v>
+        <v>1247</v>
       </c>
       <c r="K166" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L166" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M166" s="3" t="s">
         <v>24</v>
@@ -12980,13 +13001,13 @@
         <v>438</v>
       </c>
       <c r="J167" s="3" t="s">
-        <v>1250</v>
+        <v>1248</v>
       </c>
       <c r="K167" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L167" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M167" s="3" t="s">
         <v>24</v>
@@ -13204,13 +13225,13 @@
         <v>702</v>
       </c>
       <c r="J172" s="41" t="s">
-        <v>1239</v>
+        <v>1237</v>
       </c>
       <c r="K172" s="3" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="L172" s="3" t="s">
-        <v>1234</v>
+        <v>1232</v>
       </c>
       <c r="M172" s="3" t="s">
         <v>24</v>
@@ -13252,13 +13273,13 @@
         <v>705</v>
       </c>
       <c r="J173" s="93" t="s">
-        <v>1238</v>
+        <v>1236</v>
       </c>
       <c r="K173" s="3" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="L173" s="3" t="s">
-        <v>1234</v>
+        <v>1232</v>
       </c>
       <c r="M173" s="3" t="s">
         <v>24</v>
@@ -13326,7 +13347,7 @@
     </row>
     <row r="175" spans="1:19" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A175" s="45" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B175" s="44" t="s">
         <v>19</v>
@@ -13349,13 +13370,13 @@
         <v>22</v>
       </c>
       <c r="J175" s="44" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="K175" s="44" t="s">
         <v>23</v>
       </c>
       <c r="L175" s="44" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M175" s="44" t="s">
         <v>24</v>
@@ -13379,34 +13400,34 @@
     </row>
     <row r="176" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A176" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B176" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C176" s="41" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="D176" s="3" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
       <c r="F176" s="1" t="b">
         <v>1</v>
       </c>
       <c r="G176" s="1" t="s">
-        <v>1208</v>
+        <v>1206</v>
       </c>
       <c r="I176" s="3" t="s">
-        <v>1147</v>
+        <v>1145</v>
       </c>
       <c r="J176" s="3" t="s">
-        <v>1244</v>
+        <v>1242</v>
       </c>
       <c r="K176" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L176" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M176" s="3" t="s">
         <v>24</v>
@@ -13429,25 +13450,25 @@
     </row>
     <row r="177" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B177" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C177" s="41" t="s">
-        <v>1106</v>
+        <v>1104</v>
       </c>
       <c r="D177" s="3" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
       <c r="F177" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I177" s="3" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
       <c r="J177" s="97" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="M177" s="3" t="s">
         <v>24</v>
@@ -13470,7 +13491,7 @@
     </row>
     <row r="178" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B178" s="3" t="s">
         <v>19</v>
@@ -13485,16 +13506,16 @@
         <v>0</v>
       </c>
       <c r="I178" s="41" t="s">
-        <v>1150</v>
+        <v>1148</v>
       </c>
       <c r="J178" s="15" t="s">
-        <v>1237</v>
+        <v>1235</v>
       </c>
       <c r="K178" s="3" t="s">
         <v>201</v>
       </c>
       <c r="L178" s="3" t="s">
-        <v>1230</v>
+        <v>1228</v>
       </c>
       <c r="M178" s="3" t="s">
         <v>24</v>
@@ -13517,25 +13538,25 @@
     </row>
     <row r="179" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B179" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C179" s="41" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="D179" s="3" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
       <c r="F179" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I179" s="41" t="s">
-        <v>1151</v>
+        <v>1149</v>
       </c>
       <c r="J179" s="93" t="s">
-        <v>1240</v>
+        <v>1238</v>
       </c>
       <c r="M179" s="3" t="s">
         <v>24</v>
@@ -13558,25 +13579,25 @@
     </row>
     <row r="180" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B180" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C180" s="41" t="s">
-        <v>1110</v>
+        <v>1108</v>
       </c>
       <c r="D180" s="17" t="s">
-        <v>1196</v>
+        <v>1194</v>
       </c>
       <c r="F180" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I180" s="41" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="J180" s="68" t="s">
-        <v>1243</v>
+        <v>1241</v>
       </c>
       <c r="M180" s="3" t="s">
         <v>24</v>
@@ -13599,25 +13620,25 @@
     </row>
     <row r="181" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B181" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C181" s="41" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
       <c r="D181" s="41" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
       <c r="F181" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I181" s="41" t="s">
-        <v>1136</v>
+        <v>1134</v>
       </c>
       <c r="J181" s="95" t="s">
-        <v>1242</v>
+        <v>1240</v>
       </c>
       <c r="M181" s="3" t="s">
         <v>24</v>
@@ -13640,25 +13661,25 @@
     </row>
     <row r="182" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B182" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C182" s="41" t="s">
-        <v>1112</v>
+        <v>1110</v>
       </c>
       <c r="D182" s="41" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="F182" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I182" s="41" t="s">
-        <v>1137</v>
+        <v>1135</v>
       </c>
       <c r="J182" s="68" t="s">
-        <v>1186</v>
+        <v>1184</v>
       </c>
       <c r="M182" s="3" t="s">
         <v>24</v>
@@ -13681,25 +13702,25 @@
     </row>
     <row r="183" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B183" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C183" s="41" t="s">
-        <v>1113</v>
+        <v>1111</v>
       </c>
       <c r="D183" s="41" t="s">
-        <v>1130</v>
+        <v>1128</v>
       </c>
       <c r="F183" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I183" s="41" t="s">
-        <v>1138</v>
+        <v>1136</v>
       </c>
       <c r="J183" s="94" t="s">
-        <v>1241</v>
+        <v>1239</v>
       </c>
       <c r="M183" s="3" t="s">
         <v>24</v>
@@ -13722,22 +13743,22 @@
     </row>
     <row r="184" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B184" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C184" s="41" t="s">
-        <v>1114</v>
+        <v>1112</v>
       </c>
       <c r="D184" s="41" t="s">
-        <v>1131</v>
+        <v>1129</v>
       </c>
       <c r="F184" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I184" s="41" t="s">
-        <v>1139</v>
+        <v>1137</v>
       </c>
       <c r="J184" s="96"/>
       <c r="M184" s="3" t="s">
@@ -13761,31 +13782,31 @@
     </row>
     <row r="185" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B185" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C185" s="41" t="s">
-        <v>1115</v>
+        <v>1113</v>
       </c>
       <c r="D185" s="41" t="s">
-        <v>1132</v>
+        <v>1130</v>
       </c>
       <c r="F185" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I185" s="41" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
       <c r="J185" s="95">
         <v>2.5</v>
       </c>
       <c r="K185" s="98" t="s">
-        <v>1254</v>
+        <v>1252</v>
       </c>
       <c r="L185" t="s">
-        <v>1235</v>
+        <v>1233</v>
       </c>
       <c r="M185" s="3" t="s">
         <v>24</v>
@@ -13808,25 +13829,25 @@
     </row>
     <row r="186" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B186" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C186" s="41" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="D186" s="41" t="s">
-        <v>1133</v>
+        <v>1131</v>
       </c>
       <c r="F186" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I186" s="41" t="s">
-        <v>1141</v>
+        <v>1139</v>
       </c>
       <c r="J186" s="33" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="M186" s="3" t="s">
         <v>24</v>
@@ -13849,22 +13870,22 @@
     </row>
     <row r="187" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B187" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C187" s="41" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="D187" s="41" t="s">
-        <v>1135</v>
+        <v>1133</v>
       </c>
       <c r="F187" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I187" s="41" t="s">
-        <v>1142</v>
+        <v>1140</v>
       </c>
       <c r="J187" s="96"/>
       <c r="M187" s="3" t="s">
@@ -13888,22 +13909,22 @@
     </row>
     <row r="188" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B188" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C188" s="41" t="s">
-        <v>1118</v>
+        <v>1116</v>
       </c>
       <c r="D188" s="41" t="s">
-        <v>1134</v>
+        <v>1132</v>
       </c>
       <c r="F188" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I188" s="41" t="s">
-        <v>1143</v>
+        <v>1141</v>
       </c>
       <c r="J188" s="96"/>
       <c r="M188" s="3" t="s">
@@ -13927,29 +13948,29 @@
     </row>
     <row r="189" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A189" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B189" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C189" s="41" t="s">
-        <v>1119</v>
+        <v>1117</v>
       </c>
       <c r="D189" s="41" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
       <c r="F189" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I189" s="41" t="s">
-        <v>1144</v>
+        <v>1142</v>
       </c>
       <c r="J189" s="3"/>
       <c r="K189" s="3" t="s">
         <v>201</v>
       </c>
       <c r="L189" s="3" t="s">
-        <v>1230</v>
+        <v>1228</v>
       </c>
       <c r="M189" s="3" t="s">
         <v>24</v>
@@ -13972,22 +13993,22 @@
     </row>
     <row r="190" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A190" s="8" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B190" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C190" s="41" t="s">
-        <v>1120</v>
+        <v>1118</v>
       </c>
       <c r="D190" s="41" t="s">
-        <v>1145</v>
+        <v>1143</v>
       </c>
       <c r="F190" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I190" s="41" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
       <c r="J190" s="3"/>
       <c r="M190" s="3" t="s">
@@ -14034,13 +14055,13 @@
         <v>22</v>
       </c>
       <c r="J191" s="44" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="K191" s="44" t="s">
         <v>23</v>
       </c>
       <c r="L191" s="44" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M191" s="44" t="s">
         <v>24</v>
@@ -14070,7 +14091,7 @@
         <v>19</v>
       </c>
       <c r="C192" t="s">
-        <v>1096</v>
+        <v>1094</v>
       </c>
       <c r="D192" t="s">
         <v>682</v>
@@ -14079,19 +14100,19 @@
         <v>1</v>
       </c>
       <c r="G192" s="1" t="s">
-        <v>1209</v>
+        <v>1207</v>
       </c>
       <c r="I192" s="3" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
       <c r="J192" s="3" t="s">
-        <v>1252</v>
+        <v>1250</v>
       </c>
       <c r="K192" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L192" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M192" s="3" t="s">
         <v>24</v>
@@ -14132,16 +14153,16 @@
         <v>277</v>
       </c>
       <c r="I193" s="3" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
       <c r="J193" s="3" t="s">
-        <v>1249</v>
+        <v>1247</v>
       </c>
       <c r="K193" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L193" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M193" s="3" t="s">
         <v>24</v>
@@ -14170,28 +14191,28 @@
         <v>19</v>
       </c>
       <c r="C194" t="s">
-        <v>1097</v>
+        <v>1095</v>
       </c>
       <c r="D194" s="3" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
       <c r="F194" s="1" t="b">
         <v>0</v>
       </c>
       <c r="H194" s="1" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="I194" s="3" t="s">
-        <v>1147</v>
+        <v>1145</v>
       </c>
       <c r="J194" s="3" t="s">
-        <v>1244</v>
+        <v>1242</v>
       </c>
       <c r="K194" s="3" t="s">
         <v>23</v>
       </c>
       <c r="L194" s="3" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="M194" s="3" t="s">
         <v>24</v>
@@ -14229,10 +14250,10 @@
         <v>0</v>
       </c>
       <c r="I195" s="3" t="s">
-        <v>1155</v>
+        <v>1153</v>
       </c>
       <c r="J195" s="3" t="s">
-        <v>1253</v>
+        <v>1251</v>
       </c>
       <c r="M195" s="3" t="s">
         <v>24</v>
@@ -14261,26 +14282,26 @@
         <v>19</v>
       </c>
       <c r="C196" t="s">
-        <v>1197</v>
+        <v>1195</v>
       </c>
       <c r="D196" s="3" t="s">
-        <v>1166</v>
+        <v>1164</v>
       </c>
       <c r="F196" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G196" s="43"/>
       <c r="I196" s="41" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
       <c r="J196" s="93" t="s">
-        <v>1251</v>
+        <v>1249</v>
       </c>
       <c r="K196" s="3" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="L196" s="3" t="s">
-        <v>1234</v>
+        <v>1232</v>
       </c>
       <c r="M196" s="3" t="s">
         <v>24</v>
@@ -14309,20 +14330,20 @@
         <v>19</v>
       </c>
       <c r="C197" s="41" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="D197" s="3" t="s">
-        <v>1161</v>
+        <v>1159</v>
       </c>
       <c r="F197" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G197" s="43"/>
       <c r="I197" s="3" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
       <c r="J197" s="68" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="M197" s="3" t="s">
         <v>24</v>
@@ -14351,17 +14372,17 @@
         <v>19</v>
       </c>
       <c r="C198" s="41" t="s">
-        <v>1107</v>
+        <v>1105</v>
       </c>
       <c r="D198" s="41" t="s">
-        <v>1162</v>
+        <v>1160</v>
       </c>
       <c r="F198" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G198" s="43"/>
       <c r="I198" s="41" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
       <c r="J198" s="3">
         <v>4</v>
@@ -14370,7 +14391,7 @@
         <v>241</v>
       </c>
       <c r="L198" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M198" s="3" t="s">
         <v>24</v>
@@ -14399,17 +14420,17 @@
         <v>19</v>
       </c>
       <c r="C199" s="41" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="D199" s="41" t="s">
-        <v>1163</v>
+        <v>1161</v>
       </c>
       <c r="F199" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G199" s="43"/>
       <c r="I199" s="41" t="s">
-        <v>1149</v>
+        <v>1147</v>
       </c>
       <c r="J199" s="3">
         <v>50</v>
@@ -14418,7 +14439,7 @@
         <v>241</v>
       </c>
       <c r="L199" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M199" s="3" t="s">
         <v>24</v>
@@ -14447,17 +14468,17 @@
         <v>19</v>
       </c>
       <c r="C200" s="41" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
       <c r="D200" s="41" t="s">
-        <v>1164</v>
+        <v>1162</v>
       </c>
       <c r="F200" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G200" s="43"/>
       <c r="I200" s="41" t="s">
-        <v>1158</v>
+        <v>1156</v>
       </c>
       <c r="J200" s="3">
         <v>90</v>
@@ -14466,7 +14487,7 @@
         <v>241</v>
       </c>
       <c r="L200" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="M200" s="3" t="s">
         <v>24</v>
@@ -14495,17 +14516,17 @@
         <v>19</v>
       </c>
       <c r="C201" s="41" t="s">
-        <v>1123</v>
+        <v>1121</v>
       </c>
       <c r="D201" s="41" t="s">
-        <v>1165</v>
+        <v>1163</v>
       </c>
       <c r="F201" s="43" t="b">
         <v>0</v>
       </c>
       <c r="G201" s="43"/>
       <c r="I201" s="41" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
       <c r="J201" s="3" t="s">
         <v>53</v>
@@ -14514,7 +14535,7 @@
         <v>54</v>
       </c>
       <c r="L201" s="3" t="s">
-        <v>1222</v>
+        <v>1220</v>
       </c>
       <c r="M201" s="3" t="s">
         <v>24</v>
@@ -14638,7 +14659,7 @@
     <col min="23" max="23" width="26.1640625" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="36.5" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="27.5" customWidth="1"/>
     <col min="27" max="27" width="61.1640625" style="39" customWidth="1"/>
     <col min="28" max="28" width="22.83203125" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="10.6640625" bestFit="1" customWidth="1"/>
@@ -14728,25 +14749,25 @@
         <v>429</v>
       </c>
       <c r="AA1" s="79" t="s">
-        <v>1098</v>
+        <v>1096</v>
       </c>
       <c r="AB1" s="79" t="s">
         <v>102</v>
       </c>
       <c r="AC1" s="90" t="s">
-        <v>1106</v>
+        <v>1104</v>
       </c>
       <c r="AD1" s="90" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="AE1" s="80" t="s">
+        <v>1108</v>
+      </c>
+      <c r="AF1" s="80" t="s">
         <v>1110</v>
       </c>
-      <c r="AF1" s="80" t="s">
-        <v>1112</v>
-      </c>
       <c r="AG1" s="81" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="2" spans="1:33" ht="16" x14ac:dyDescent="0.2">
@@ -14820,7 +14841,7 @@
         <v>724</v>
       </c>
       <c r="X2" s="36" t="s">
-        <v>725</v>
+        <v>826</v>
       </c>
       <c r="Y2" s="36" t="s">
         <v>726</v>
@@ -14832,22 +14853,22 @@
         <v>728</v>
       </c>
       <c r="AB2" s="36" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
       <c r="AC2" s="73" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="AD2" s="74" t="s">
-        <v>1173</v>
+        <v>1171</v>
       </c>
       <c r="AE2" s="73" t="s">
-        <v>1178</v>
+        <v>1176</v>
       </c>
       <c r="AF2" s="73" t="s">
-        <v>1183</v>
+        <v>1181</v>
       </c>
       <c r="AG2" s="74" t="s">
-        <v>1189</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="3" spans="1:33" ht="16" x14ac:dyDescent="0.2">
@@ -14921,34 +14942,34 @@
         <v>742</v>
       </c>
       <c r="X3" s="36" t="s">
-        <v>743</v>
+        <v>725</v>
       </c>
       <c r="Y3" s="36" t="s">
         <v>295</v>
       </c>
-      <c r="Z3" s="68" t="s">
-        <v>744</v>
+      <c r="Z3" s="36" t="s">
+        <v>1263</v>
       </c>
       <c r="AA3" s="69" t="s">
         <v>745</v>
       </c>
       <c r="AB3" s="36" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
       <c r="AC3" s="36" t="s">
-        <v>1168</v>
+        <v>1166</v>
       </c>
       <c r="AD3" s="70" t="s">
-        <v>1174</v>
+        <v>1172</v>
       </c>
       <c r="AE3" s="36" t="s">
-        <v>1179</v>
+        <v>1177</v>
       </c>
       <c r="AF3" s="36" t="s">
-        <v>1184</v>
+        <v>1182</v>
       </c>
       <c r="AG3" s="70" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="4" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.2">
@@ -15010,34 +15031,34 @@
         <v>758</v>
       </c>
       <c r="X4" s="36" t="s">
-        <v>759</v>
+        <v>743</v>
       </c>
       <c r="Y4" s="36" t="s">
         <v>760</v>
       </c>
       <c r="Z4" s="68" t="s">
-        <v>761</v>
+        <v>744</v>
       </c>
       <c r="AA4" s="69" t="s">
         <v>762</v>
       </c>
       <c r="AB4" s="36" t="s">
-        <v>1104</v>
+        <v>1102</v>
       </c>
       <c r="AC4" s="36" t="s">
-        <v>1169</v>
+        <v>1167</v>
       </c>
       <c r="AD4" s="35" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="AE4" s="36" t="s">
-        <v>1180</v>
+        <v>1178</v>
       </c>
       <c r="AF4" s="36" t="s">
-        <v>1185</v>
+        <v>1183</v>
       </c>
       <c r="AG4" s="35" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="5" spans="1:33" ht="16" x14ac:dyDescent="0.2">
@@ -15093,34 +15114,34 @@
         <v>773</v>
       </c>
       <c r="X5" s="36" t="s">
-        <v>774</v>
+        <v>759</v>
       </c>
       <c r="Y5" s="36" t="s">
         <v>775</v>
       </c>
-      <c r="Z5" s="68" t="s">
-        <v>776</v>
+      <c r="Z5" s="36" t="s">
+        <v>1264</v>
       </c>
       <c r="AA5" s="69" t="s">
         <v>777</v>
       </c>
       <c r="AB5" s="36" t="s">
-        <v>1101</v>
+        <v>1099</v>
       </c>
       <c r="AC5" s="36" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
       <c r="AD5" s="35" t="s">
-        <v>1176</v>
+        <v>1174</v>
       </c>
       <c r="AE5" s="36" t="s">
-        <v>1181</v>
+        <v>1179</v>
       </c>
       <c r="AF5" s="36" t="s">
-        <v>1186</v>
+        <v>1184</v>
       </c>
       <c r="AG5" s="35" t="s">
-        <v>1192</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="6" spans="1:33" ht="16" x14ac:dyDescent="0.2">
@@ -15172,28 +15193,28 @@
         <v>787</v>
       </c>
       <c r="Z6" s="68" t="s">
-        <v>788</v>
+        <v>761</v>
       </c>
       <c r="AA6" s="69" t="s">
         <v>789</v>
       </c>
       <c r="AB6" s="36" t="s">
-        <v>1102</v>
+        <v>1100</v>
       </c>
       <c r="AC6" s="36" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="AD6" s="36" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="AE6" s="36" t="s">
-        <v>1182</v>
+        <v>1180</v>
       </c>
       <c r="AF6" s="36" t="s">
-        <v>1187</v>
+        <v>1185</v>
       </c>
       <c r="AG6" s="35" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="7" spans="1:33" ht="16" x14ac:dyDescent="0.2">
@@ -15233,30 +15254,30 @@
         <v>796</v>
       </c>
       <c r="X7" s="36" t="s">
-        <v>797</v>
+        <v>774</v>
       </c>
       <c r="Y7" s="36" t="s">
         <v>798</v>
       </c>
       <c r="Z7" s="68" t="s">
-        <v>799</v>
+        <v>776</v>
       </c>
       <c r="AA7" s="69" t="s">
         <v>105</v>
       </c>
       <c r="AB7" s="36" t="s">
-        <v>1103</v>
+        <v>1101</v>
       </c>
       <c r="AC7" s="36" t="s">
-        <v>1172</v>
+        <v>1170</v>
       </c>
       <c r="AD7" s="36"/>
       <c r="AE7" s="36"/>
       <c r="AF7" s="36" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="AG7" s="35" t="s">
-        <v>1194</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="8" spans="1:33" ht="16" x14ac:dyDescent="0.2">
@@ -15294,13 +15315,13 @@
         <v>804</v>
       </c>
       <c r="X8" s="36" t="s">
-        <v>805</v>
+        <v>797</v>
       </c>
       <c r="Y8" s="36" t="s">
         <v>806</v>
       </c>
       <c r="Z8" s="68" t="s">
-        <v>807</v>
+        <v>788</v>
       </c>
       <c r="AA8" s="69"/>
       <c r="AB8" s="36"/>
@@ -15343,12 +15364,14 @@
         <v>811</v>
       </c>
       <c r="X9" s="36" t="s">
-        <v>812</v>
+        <v>805</v>
       </c>
       <c r="Y9" s="36" t="s">
         <v>813</v>
       </c>
-      <c r="Z9" s="36"/>
+      <c r="Z9" s="68" t="s">
+        <v>799</v>
+      </c>
       <c r="AA9" s="69"/>
       <c r="AB9" s="36"/>
       <c r="AC9" s="36"/>
@@ -15386,12 +15409,14 @@
         <v>815</v>
       </c>
       <c r="X10" s="36" t="s">
-        <v>816</v>
+        <v>812</v>
       </c>
       <c r="Y10" s="36" t="s">
         <v>817</v>
       </c>
-      <c r="Z10" s="36"/>
+      <c r="Z10" s="68" t="s">
+        <v>807</v>
+      </c>
       <c r="AA10" s="69"/>
       <c r="AB10" s="36"/>
       <c r="AC10" s="36"/>
@@ -15429,7 +15454,7 @@
         <v>819</v>
       </c>
       <c r="X11" s="36" t="s">
-        <v>820</v>
+        <v>816</v>
       </c>
       <c r="Y11" s="36" t="s">
         <v>821</v>
@@ -15470,10 +15495,10 @@
         <v>822</v>
       </c>
       <c r="X12" s="36" t="s">
-        <v>823</v>
+        <v>820</v>
       </c>
       <c r="Y12" s="36" t="s">
-        <v>824</v>
+        <v>1265</v>
       </c>
       <c r="Z12" s="36"/>
       <c r="AA12" s="69"/>
@@ -15511,10 +15536,10 @@
         <v>825</v>
       </c>
       <c r="X13" s="36" t="s">
-        <v>826</v>
+        <v>823</v>
       </c>
       <c r="Y13" s="36" t="s">
-        <v>827</v>
+        <v>1267</v>
       </c>
       <c r="Z13" s="36"/>
       <c r="AA13" s="69"/>
@@ -15549,13 +15574,13 @@
       <c r="U14" s="36"/>
       <c r="V14" s="36"/>
       <c r="W14" s="36" t="s">
+        <v>827</v>
+      </c>
+      <c r="X14" s="36" t="s">
         <v>828</v>
       </c>
-      <c r="X14" s="36" t="s">
-        <v>829</v>
-      </c>
       <c r="Y14" s="36" t="s">
-        <v>830</v>
+        <v>1266</v>
       </c>
       <c r="Z14" s="36"/>
       <c r="AA14" s="69"/>
@@ -15590,13 +15615,13 @@
       <c r="U15" s="36"/>
       <c r="V15" s="36"/>
       <c r="W15" s="36" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
       <c r="X15" s="36" t="s">
-        <v>832</v>
+        <v>830</v>
       </c>
       <c r="Y15" s="36" t="s">
-        <v>833</v>
+        <v>675</v>
       </c>
       <c r="Z15" s="36"/>
       <c r="AA15" s="69"/>
@@ -15631,13 +15656,13 @@
       <c r="U16" s="36"/>
       <c r="V16" s="36"/>
       <c r="W16" s="36" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="X16" s="36" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="Y16" s="36" t="s">
-        <v>836</v>
+        <v>1268</v>
       </c>
       <c r="Z16" s="36"/>
       <c r="AA16" s="69"/>
@@ -15672,13 +15697,13 @@
       <c r="U17" s="36"/>
       <c r="V17" s="36"/>
       <c r="W17" s="36" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
       <c r="X17" s="36" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
       <c r="Y17" s="36" t="s">
-        <v>839</v>
+        <v>859</v>
       </c>
       <c r="Z17" s="36"/>
       <c r="AA17" s="69"/>
@@ -15713,13 +15738,13 @@
       <c r="U18" s="36"/>
       <c r="V18" s="36"/>
       <c r="W18" s="36" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="X18" s="36" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
       <c r="Y18" s="36" t="s">
-        <v>842</v>
+        <v>824</v>
       </c>
       <c r="Z18" s="36"/>
       <c r="AA18" s="69"/>
@@ -15754,13 +15779,13 @@
       <c r="U19" s="36"/>
       <c r="V19" s="36"/>
       <c r="W19" s="36" t="s">
-        <v>843</v>
+        <v>841</v>
       </c>
       <c r="X19" s="36" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="Y19" s="36" t="s">
-        <v>845</v>
+        <v>848</v>
       </c>
       <c r="Z19" s="36"/>
       <c r="AA19" s="69"/>
@@ -15795,13 +15820,13 @@
       <c r="U20" s="36"/>
       <c r="V20" s="36"/>
       <c r="W20" s="36" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
       <c r="X20" s="36" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
       <c r="Y20" s="36" t="s">
-        <v>848</v>
+        <v>1269</v>
       </c>
       <c r="Z20" s="36"/>
       <c r="AA20" s="69"/>
@@ -15836,13 +15861,13 @@
       <c r="U21" s="36"/>
       <c r="V21" s="36"/>
       <c r="W21" s="36" t="s">
-        <v>849</v>
+        <v>847</v>
       </c>
       <c r="X21" s="36" t="s">
-        <v>850</v>
+        <v>848</v>
       </c>
       <c r="Y21" s="36" t="s">
-        <v>851</v>
+        <v>1270</v>
       </c>
       <c r="Z21" s="36"/>
       <c r="AA21" s="69"/>
@@ -15877,13 +15902,13 @@
       <c r="U22" s="36"/>
       <c r="V22" s="36"/>
       <c r="W22" s="36" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="X22" s="36" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
       <c r="Y22" s="36" t="s">
-        <v>854</v>
+        <v>831</v>
       </c>
       <c r="Z22" s="36"/>
       <c r="AA22" s="69"/>
@@ -15918,13 +15943,13 @@
       <c r="U23" s="36"/>
       <c r="V23" s="36"/>
       <c r="W23" s="36" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
       <c r="X23" s="36" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
       <c r="Y23" s="36" t="s">
-        <v>857</v>
+        <v>834</v>
       </c>
       <c r="Z23" s="36"/>
       <c r="AA23" s="71"/>
@@ -15962,10 +15987,10 @@
         <v>449</v>
       </c>
       <c r="X24" s="36" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="Y24" s="36" t="s">
-        <v>675</v>
+        <v>837</v>
       </c>
       <c r="Z24" s="36"/>
       <c r="AA24" s="69"/>
@@ -16000,13 +16025,13 @@
       <c r="U25" s="36"/>
       <c r="V25" s="36"/>
       <c r="W25" s="36" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
       <c r="X25" s="36" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="Y25" s="36" t="s">
-        <v>861</v>
+        <v>840</v>
       </c>
       <c r="Z25" s="36"/>
       <c r="AA25" s="69"/>
@@ -16041,13 +16066,13 @@
       <c r="U26" s="36"/>
       <c r="V26" s="36"/>
       <c r="W26" s="36" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="X26" s="36" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="Y26" s="36" t="s">
-        <v>850</v>
+        <v>843</v>
       </c>
       <c r="Z26" s="36"/>
       <c r="AA26" s="69"/>
@@ -16082,13 +16107,13 @@
       <c r="U27" s="36"/>
       <c r="V27" s="36"/>
       <c r="W27" s="36" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="X27" s="36" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="Y27" s="36" t="s">
-        <v>866</v>
+        <v>846</v>
       </c>
       <c r="Z27" s="36"/>
       <c r="AA27" s="69"/>
@@ -16123,13 +16148,13 @@
       <c r="U28" s="36"/>
       <c r="V28" s="36"/>
       <c r="W28" s="36" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="X28" s="36" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="Y28" s="36" t="s">
-        <v>869</v>
+        <v>849</v>
       </c>
       <c r="Z28" s="36"/>
       <c r="AA28" s="69"/>
@@ -16164,12 +16189,14 @@
       <c r="U29" s="36"/>
       <c r="V29" s="36"/>
       <c r="W29" s="36" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="X29" s="36" t="s">
-        <v>871</v>
-      </c>
-      <c r="Y29" s="36"/>
+        <v>869</v>
+      </c>
+      <c r="Y29" s="36" t="s">
+        <v>852</v>
+      </c>
       <c r="Z29" s="36"/>
       <c r="AA29" s="69"/>
       <c r="AB29" s="36"/>
@@ -16203,12 +16230,14 @@
       <c r="U30" s="36"/>
       <c r="V30" s="36"/>
       <c r="W30" s="36" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="X30" s="36" t="s">
-        <v>873</v>
-      </c>
-      <c r="Y30" s="36"/>
+        <v>871</v>
+      </c>
+      <c r="Y30" s="36" t="s">
+        <v>855</v>
+      </c>
       <c r="Z30" s="36"/>
       <c r="AA30" s="69"/>
       <c r="AB30" s="36"/>
@@ -16242,12 +16271,14 @@
       <c r="U31" s="36"/>
       <c r="V31" s="36"/>
       <c r="W31" s="36" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
       <c r="X31" s="36" t="s">
-        <v>875</v>
-      </c>
-      <c r="Y31" s="36"/>
+        <v>873</v>
+      </c>
+      <c r="Y31" s="36" t="s">
+        <v>864</v>
+      </c>
       <c r="Z31" s="36"/>
       <c r="AA31" s="69"/>
       <c r="AB31" s="36"/>
@@ -16281,12 +16312,14 @@
       <c r="U32" s="36"/>
       <c r="V32" s="36"/>
       <c r="W32" s="36" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
       <c r="X32" s="36" t="s">
-        <v>877</v>
-      </c>
-      <c r="Y32" s="36"/>
+        <v>875</v>
+      </c>
+      <c r="Y32" s="36" t="s">
+        <v>867</v>
+      </c>
       <c r="Z32" s="36"/>
       <c r="AA32" s="69"/>
       <c r="AB32" s="36"/>
@@ -16320,10 +16353,10 @@
       <c r="U33" s="36"/>
       <c r="V33" s="36"/>
       <c r="W33" s="36" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
       <c r="X33" s="36" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="Y33" s="36"/>
       <c r="Z33" s="36"/>
@@ -16359,10 +16392,10 @@
       <c r="U34" s="36"/>
       <c r="V34" s="36"/>
       <c r="W34" s="36" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
       <c r="X34" s="36" t="s">
-        <v>881</v>
+        <v>879</v>
       </c>
       <c r="Y34" s="36"/>
       <c r="Z34" s="36"/>
@@ -16398,10 +16431,10 @@
       <c r="U35" s="36"/>
       <c r="V35" s="36"/>
       <c r="W35" s="36" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
       <c r="X35" s="36" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="Y35" s="36"/>
       <c r="Z35" s="36"/>
@@ -16437,10 +16470,10 @@
       <c r="U36" s="36"/>
       <c r="V36" s="36"/>
       <c r="W36" s="36" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="X36" s="36" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="Y36" s="36"/>
       <c r="Z36" s="36"/>
@@ -16476,10 +16509,10 @@
       <c r="U37" s="36"/>
       <c r="V37" s="36"/>
       <c r="W37" s="36" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="X37" s="36" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
       <c r="Y37" s="36"/>
       <c r="Z37" s="36"/>
@@ -16515,10 +16548,10 @@
       <c r="U38" s="36"/>
       <c r="V38" s="36"/>
       <c r="W38" s="36" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
       <c r="X38" s="36" t="s">
-        <v>889</v>
+        <v>1271</v>
       </c>
       <c r="Y38" s="36"/>
       <c r="Z38" s="36"/>
@@ -16554,10 +16587,10 @@
       <c r="U39" s="36"/>
       <c r="V39" s="36"/>
       <c r="W39" s="36" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
       <c r="X39" s="36" t="s">
-        <v>891</v>
+        <v>887</v>
       </c>
       <c r="Y39" s="36"/>
       <c r="Z39" s="36"/>
@@ -16593,10 +16626,10 @@
       <c r="U40" s="36"/>
       <c r="V40" s="36"/>
       <c r="W40" s="36" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
       <c r="X40" s="36" t="s">
-        <v>893</v>
+        <v>889</v>
       </c>
       <c r="Y40" s="36"/>
       <c r="Z40" s="36"/>
@@ -16632,10 +16665,10 @@
       <c r="U41" s="36"/>
       <c r="V41" s="36"/>
       <c r="W41" s="36" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
       <c r="X41" s="36" t="s">
-        <v>807</v>
+        <v>891</v>
       </c>
       <c r="Y41" s="36"/>
       <c r="Z41" s="36"/>
@@ -16671,9 +16704,11 @@
       <c r="U42" s="36"/>
       <c r="V42" s="36"/>
       <c r="W42" s="36" t="s">
-        <v>895</v>
-      </c>
-      <c r="X42" s="36"/>
+        <v>893</v>
+      </c>
+      <c r="X42" s="36" t="s">
+        <v>807</v>
+      </c>
       <c r="Y42" s="36"/>
       <c r="Z42" s="36"/>
       <c r="AA42" s="69"/>
@@ -16708,7 +16743,7 @@
       <c r="U43" s="36"/>
       <c r="V43" s="36"/>
       <c r="W43" s="36" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="X43" s="36"/>
       <c r="Y43" s="36"/>
@@ -16745,7 +16780,7 @@
       <c r="U44" s="36"/>
       <c r="V44" s="36"/>
       <c r="W44" s="36" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
       <c r="X44" s="36"/>
       <c r="Y44" s="36"/>
@@ -16782,7 +16817,7 @@
       <c r="U45" s="36"/>
       <c r="V45" s="36"/>
       <c r="W45" s="36" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="X45" s="36"/>
       <c r="Y45" s="36"/>
@@ -16819,7 +16854,7 @@
       <c r="U46" s="36"/>
       <c r="V46" s="36"/>
       <c r="W46" s="36" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="X46" s="36"/>
       <c r="Y46" s="36"/>
@@ -16856,7 +16891,7 @@
       <c r="U47" s="36"/>
       <c r="V47" s="36"/>
       <c r="W47" s="36" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="X47" s="36"/>
       <c r="Y47" s="36"/>
@@ -16893,7 +16928,7 @@
       <c r="U48" s="36"/>
       <c r="V48" s="36"/>
       <c r="W48" s="36" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="X48" s="36"/>
       <c r="Y48" s="36"/>
@@ -16930,7 +16965,7 @@
       <c r="U49" s="36"/>
       <c r="V49" s="36"/>
       <c r="W49" s="36" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
       <c r="X49" s="36"/>
       <c r="Y49" s="36"/>
@@ -16967,7 +17002,7 @@
       <c r="U50" s="36"/>
       <c r="V50" s="36"/>
       <c r="W50" s="36" t="s">
-        <v>903</v>
+        <v>901</v>
       </c>
       <c r="X50" s="36"/>
       <c r="Y50" s="36"/>
@@ -17004,7 +17039,7 @@
       <c r="U51" s="36"/>
       <c r="V51" s="36"/>
       <c r="W51" s="36" t="s">
-        <v>904</v>
+        <v>902</v>
       </c>
       <c r="X51" s="36"/>
       <c r="Y51" s="36"/>
@@ -17041,7 +17076,7 @@
       <c r="U52" s="36"/>
       <c r="V52" s="36"/>
       <c r="W52" s="36" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="X52" s="36"/>
       <c r="Y52" s="36"/>
@@ -17078,7 +17113,7 @@
       <c r="U53" s="36"/>
       <c r="V53" s="36"/>
       <c r="W53" s="36" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="X53" s="36"/>
       <c r="Y53" s="36"/>
@@ -17115,7 +17150,7 @@
       <c r="U54" s="36"/>
       <c r="V54" s="36"/>
       <c r="W54" s="36" t="s">
-        <v>907</v>
+        <v>905</v>
       </c>
       <c r="X54" s="36"/>
       <c r="Y54" s="36"/>
@@ -17152,7 +17187,7 @@
       <c r="U55" s="36"/>
       <c r="V55" s="36"/>
       <c r="W55" s="36" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="X55" s="36"/>
       <c r="Y55" s="36"/>
@@ -17189,7 +17224,7 @@
       <c r="U56" s="36"/>
       <c r="V56" s="36"/>
       <c r="W56" s="36" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
       <c r="X56" s="36"/>
       <c r="Y56" s="36"/>
@@ -17226,7 +17261,7 @@
       <c r="U57" s="36"/>
       <c r="V57" s="36"/>
       <c r="W57" s="36" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="X57" s="36"/>
       <c r="Y57" s="36"/>
@@ -17263,7 +17298,7 @@
       <c r="U58" s="36"/>
       <c r="V58" s="36"/>
       <c r="W58" s="36" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
       <c r="X58" s="36"/>
       <c r="Y58" s="36"/>
@@ -17300,7 +17335,7 @@
       <c r="U59" s="36"/>
       <c r="V59" s="36"/>
       <c r="W59" s="36" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="X59" s="36"/>
       <c r="Y59" s="36"/>
@@ -17337,7 +17372,7 @@
       <c r="U60" s="36"/>
       <c r="V60" s="36"/>
       <c r="W60" s="36" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
       <c r="X60" s="36"/>
       <c r="Y60" s="36"/>
@@ -17374,7 +17409,7 @@
       <c r="U61" s="36"/>
       <c r="V61" s="36"/>
       <c r="W61" s="36" t="s">
-        <v>914</v>
+        <v>912</v>
       </c>
       <c r="X61" s="36"/>
       <c r="Y61" s="36"/>
@@ -17411,7 +17446,7 @@
       <c r="U62" s="36"/>
       <c r="V62" s="36"/>
       <c r="W62" s="36" t="s">
-        <v>915</v>
+        <v>913</v>
       </c>
       <c r="X62" s="36"/>
       <c r="Y62" s="36"/>
@@ -17448,7 +17483,7 @@
       <c r="U63" s="36"/>
       <c r="V63" s="36"/>
       <c r="W63" s="36" t="s">
-        <v>916</v>
+        <v>914</v>
       </c>
       <c r="X63" s="36"/>
       <c r="Y63" s="36"/>
@@ -17485,7 +17520,7 @@
       <c r="U64" s="36"/>
       <c r="V64" s="36"/>
       <c r="W64" s="36" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
       <c r="X64" s="36"/>
       <c r="Y64" s="36"/>
@@ -17522,7 +17557,7 @@
       <c r="U65" s="36"/>
       <c r="V65" s="36"/>
       <c r="W65" s="36" t="s">
-        <v>918</v>
+        <v>916</v>
       </c>
       <c r="X65" s="36"/>
       <c r="Y65" s="36"/>
@@ -17559,7 +17594,7 @@
       <c r="U66" s="36"/>
       <c r="V66" s="36"/>
       <c r="W66" s="36" t="s">
-        <v>919</v>
+        <v>917</v>
       </c>
       <c r="X66" s="36"/>
       <c r="Y66" s="36"/>
@@ -17596,7 +17631,7 @@
       <c r="U67" s="36"/>
       <c r="V67" s="36"/>
       <c r="W67" s="36" t="s">
-        <v>920</v>
+        <v>918</v>
       </c>
       <c r="X67" s="36"/>
       <c r="Y67" s="36"/>
@@ -17633,7 +17668,7 @@
       <c r="U68" s="36"/>
       <c r="V68" s="36"/>
       <c r="W68" s="36" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
       <c r="X68" s="36"/>
       <c r="Y68" s="36"/>
@@ -17670,7 +17705,7 @@
       <c r="U69" s="36"/>
       <c r="V69" s="36"/>
       <c r="W69" s="36" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
       <c r="X69" s="36"/>
       <c r="Y69" s="36"/>
@@ -17707,7 +17742,7 @@
       <c r="U70" s="36"/>
       <c r="V70" s="36"/>
       <c r="W70" s="36" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
       <c r="X70" s="36"/>
       <c r="Y70" s="36"/>
@@ -17744,7 +17779,7 @@
       <c r="U71" s="36"/>
       <c r="V71" s="36"/>
       <c r="W71" s="36" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="X71" s="36"/>
       <c r="Y71" s="36"/>
@@ -17781,7 +17816,7 @@
       <c r="U72" s="36"/>
       <c r="V72" s="36"/>
       <c r="W72" s="36" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="X72" s="36"/>
       <c r="Y72" s="36"/>
@@ -17818,7 +17853,7 @@
       <c r="U73" s="36"/>
       <c r="V73" s="36"/>
       <c r="W73" s="36" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
       <c r="X73" s="36"/>
       <c r="Y73" s="36"/>
@@ -17855,7 +17890,7 @@
       <c r="U74" s="36"/>
       <c r="V74" s="36"/>
       <c r="W74" s="36" t="s">
-        <v>927</v>
+        <v>925</v>
       </c>
       <c r="X74" s="36"/>
       <c r="Y74" s="36"/>
@@ -17892,7 +17927,7 @@
       <c r="U75" s="36"/>
       <c r="V75" s="36"/>
       <c r="W75" s="36" t="s">
-        <v>928</v>
+        <v>926</v>
       </c>
       <c r="X75" s="36"/>
       <c r="Y75" s="36"/>
@@ -17929,7 +17964,7 @@
       <c r="U76" s="36"/>
       <c r="V76" s="36"/>
       <c r="W76" s="36" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="X76" s="36"/>
       <c r="Y76" s="36"/>
@@ -17966,7 +18001,7 @@
       <c r="U77" s="36"/>
       <c r="V77" s="36"/>
       <c r="W77" s="36" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="X77" s="36"/>
       <c r="Y77" s="36"/>
@@ -18003,7 +18038,7 @@
       <c r="U78" s="36"/>
       <c r="V78" s="36"/>
       <c r="W78" s="36" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
       <c r="X78" s="36"/>
       <c r="Y78" s="36"/>
@@ -18040,7 +18075,7 @@
       <c r="U79" s="36"/>
       <c r="V79" s="36"/>
       <c r="W79" s="36" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
       <c r="X79" s="36"/>
       <c r="Y79" s="36"/>
@@ -18077,7 +18112,7 @@
       <c r="U80" s="36"/>
       <c r="V80" s="36"/>
       <c r="W80" s="36" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="X80" s="36"/>
       <c r="Y80" s="36"/>
@@ -18114,7 +18149,7 @@
       <c r="U81" s="36"/>
       <c r="V81" s="36"/>
       <c r="W81" s="36" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
       <c r="X81" s="36"/>
       <c r="Y81" s="36"/>
@@ -18151,7 +18186,7 @@
       <c r="U82" s="36"/>
       <c r="V82" s="36"/>
       <c r="W82" s="36" t="s">
-        <v>935</v>
+        <v>933</v>
       </c>
       <c r="X82" s="36"/>
       <c r="Y82" s="36"/>
@@ -18188,7 +18223,7 @@
       <c r="U83" s="36"/>
       <c r="V83" s="36"/>
       <c r="W83" s="36" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
       <c r="X83" s="36"/>
       <c r="Y83" s="36"/>
@@ -18225,7 +18260,7 @@
       <c r="U84" s="36"/>
       <c r="V84" s="36"/>
       <c r="W84" s="36" t="s">
-        <v>937</v>
+        <v>935</v>
       </c>
       <c r="X84" s="36"/>
       <c r="Y84" s="36"/>
@@ -26192,16 +26227,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>40</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>61</v>
@@ -26212,16 +26247,16 @@
         <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>1211</v>
+        <v>1209</v>
       </c>
       <c r="C2" t="s">
-        <v>1212</v>
+        <v>1210</v>
       </c>
       <c r="D2" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="E2" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -26229,16 +26264,16 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>1213</v>
+        <v>1211</v>
       </c>
       <c r="C3" t="s">
-        <v>1214</v>
+        <v>1212</v>
       </c>
       <c r="D3" t="s">
         <v>35</v>
       </c>
       <c r="E3" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -26246,16 +26281,16 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>1215</v>
+        <v>1213</v>
       </c>
       <c r="C4" t="s">
-        <v>1216</v>
+        <v>1214</v>
       </c>
       <c r="D4" t="s">
         <v>242</v>
       </c>
       <c r="E4" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -26263,16 +26298,16 @@
         <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>1217</v>
+        <v>1215</v>
       </c>
       <c r="C5" t="s">
-        <v>1218</v>
+        <v>1216</v>
       </c>
       <c r="D5" t="s">
         <v>89</v>
       </c>
       <c r="E5" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
     </row>
   </sheetData>
@@ -26296,16 +26331,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>943</v>
+        <v>941</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>944</v>
+        <v>942</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -26313,7 +26348,7 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
       <c r="C2" t="s">
         <v>18</v>
@@ -26327,7 +26362,7 @@
         <v>106</v>
       </c>
       <c r="B3" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -26343,7 +26378,7 @@
         <v>170</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>947</v>
+        <v>945</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -26351,7 +26386,7 @@
         <v>226</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -26359,7 +26394,7 @@
         <v>277</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -26367,7 +26402,7 @@
         <v>435</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -26375,7 +26410,7 @@
         <v>514</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -26383,7 +26418,7 @@
         <v>530</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -26391,7 +26426,7 @@
         <v>631</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -26399,7 +26434,7 @@
         <v>642</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -26407,18 +26442,18 @@
         <v>519</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="C13" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="45" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1195</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="17" thickTop="1" x14ac:dyDescent="0.2">
@@ -26448,10 +26483,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="16" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>957</v>
+        <v>955</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -26461,12 +26496,12 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
     </row>
   </sheetData>
@@ -26494,10 +26529,10 @@
         <v>9</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
       <c r="C1" s="20" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -26505,21 +26540,21 @@
         <v>23</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="21" t="s">
+        <v>962</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>963</v>
+      </c>
+      <c r="C3" s="22" t="s">
         <v>964</v>
-      </c>
-      <c r="B3" s="21" t="s">
-        <v>965</v>
-      </c>
-      <c r="C3" s="22" t="s">
-        <v>966</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -26527,43 +26562,43 @@
         <v>129</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>967</v>
+        <v>965</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>968</v>
+        <v>966</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="21" t="s">
+        <v>967</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>968</v>
+      </c>
+      <c r="C5" s="22" t="s">
         <v>969</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>970</v>
-      </c>
-      <c r="C5" s="22" t="s">
-        <v>971</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="21" t="s">
+        <v>970</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>971</v>
+      </c>
+      <c r="C6" s="22" t="s">
         <v>972</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>973</v>
-      </c>
-      <c r="C6" s="22" t="s">
-        <v>974</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="21" t="s">
+        <v>973</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>974</v>
+      </c>
+      <c r="C7" s="22" t="s">
         <v>975</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>976</v>
-      </c>
-      <c r="C7" s="22" t="s">
-        <v>977</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -26571,7 +26606,7 @@
         <v>80</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
       <c r="C8" s="22"/>
     </row>
@@ -26580,16 +26615,16 @@
         <v>98</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
       <c r="C9" s="22"/>
     </row>
     <row r="10" spans="1:3" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="21" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>981</v>
+        <v>979</v>
       </c>
       <c r="C10" s="22"/>
     </row>
@@ -26598,63 +26633,63 @@
         <v>241</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="21" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="C12" s="22"/>
     </row>
     <row r="13" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="21" t="s">
+        <v>984</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>985</v>
+      </c>
+      <c r="C13" s="22" t="s">
         <v>986</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>987</v>
-      </c>
-      <c r="C13" s="22" t="s">
-        <v>988</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="21" t="s">
+        <v>987</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>988</v>
+      </c>
+      <c r="C14" s="22" t="s">
         <v>989</v>
-      </c>
-      <c r="B14" s="21" t="s">
-        <v>990</v>
-      </c>
-      <c r="C14" s="22" t="s">
-        <v>991</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="21" t="s">
+        <v>990</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>991</v>
+      </c>
+      <c r="C15" s="22" t="s">
         <v>992</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>993</v>
-      </c>
-      <c r="C15" s="22" t="s">
-        <v>994</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="21" t="s">
+        <v>993</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>994</v>
+      </c>
+      <c r="C16" s="22" t="s">
         <v>995</v>
-      </c>
-      <c r="B16" s="21" t="s">
-        <v>996</v>
-      </c>
-      <c r="C16" s="22" t="s">
-        <v>997</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -26662,21 +26697,21 @@
         <v>676</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>998</v>
+        <v>996</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>999</v>
+        <v>997</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="21" t="s">
+        <v>998</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>999</v>
+      </c>
+      <c r="C18" s="22" t="s">
         <v>1000</v>
-      </c>
-      <c r="B18" s="21" t="s">
-        <v>1001</v>
-      </c>
-      <c r="C18" s="22" t="s">
-        <v>1002</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -26684,25 +26719,25 @@
         <v>390</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>1003</v>
+        <v>1001</v>
       </c>
       <c r="C19" s="22"/>
     </row>
     <row r="20" spans="1:3" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="17" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>1005</v>
+        <v>1003</v>
       </c>
       <c r="C20" s="22"/>
     </row>
     <row r="21" spans="1:3" ht="41.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="21" t="s">
-        <v>1006</v>
+        <v>1004</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>1007</v>
+        <v>1005</v>
       </c>
       <c r="C21" s="22"/>
     </row>
@@ -26711,41 +26746,41 @@
         <v>379</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>1008</v>
+        <v>1006</v>
       </c>
       <c r="C22" s="22"/>
     </row>
     <row r="23" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="21" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>1008</v>
+      </c>
+      <c r="C23" s="22" t="s">
         <v>1009</v>
-      </c>
-      <c r="B23" s="21" t="s">
-        <v>1010</v>
-      </c>
-      <c r="C23" s="22" t="s">
-        <v>1011</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="21" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B24" s="21" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C24" s="22" t="s">
         <v>1012</v>
-      </c>
-      <c r="B24" s="21" t="s">
-        <v>1013</v>
-      </c>
-      <c r="C24" s="22" t="s">
-        <v>1014</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="41.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="21" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C25" s="22" t="s">
         <v>1015</v>
-      </c>
-      <c r="B25" s="21" t="s">
-        <v>1016</v>
-      </c>
-      <c r="C25" s="22" t="s">
-        <v>1017</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -26753,10 +26788,10 @@
         <v>201</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>1018</v>
+        <v>1016</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -26764,10 +26799,10 @@
         <v>400</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>1020</v>
+        <v>1018</v>
       </c>
       <c r="C27" s="22" t="s">
-        <v>1021</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -26775,10 +26810,10 @@
         <v>54</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>1022</v>
+        <v>1020</v>
       </c>
       <c r="C28" s="22" t="s">
-        <v>1023</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -26786,10 +26821,10 @@
         <v>614</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -26797,43 +26832,43 @@
         <v>677</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="21" t="s">
+        <v>1026</v>
+      </c>
+      <c r="B31" s="21" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C31" s="22" t="s">
         <v>1028</v>
-      </c>
-      <c r="B31" s="21" t="s">
-        <v>1029</v>
-      </c>
-      <c r="C31" s="22" t="s">
-        <v>1030</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="17" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B32" s="21" t="s">
+        <v>1030</v>
+      </c>
+      <c r="C32" s="22" t="s">
         <v>1031</v>
-      </c>
-      <c r="B32" s="21" t="s">
-        <v>1032</v>
-      </c>
-      <c r="C32" s="22" t="s">
-        <v>1033</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="21" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B33" s="21" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C33" s="22" t="s">
         <v>1034</v>
-      </c>
-      <c r="B33" s="21" t="s">
-        <v>1035</v>
-      </c>
-      <c r="C33" s="22" t="s">
-        <v>1036</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.2">
@@ -26841,21 +26876,21 @@
         <v>111</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="26" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B35" s="26" t="s">
+        <v>1038</v>
+      </c>
+      <c r="C35" s="27" t="s">
         <v>1039</v>
-      </c>
-      <c r="B35" s="26" t="s">
-        <v>1040</v>
-      </c>
-      <c r="C35" s="27" t="s">
-        <v>1041</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -26863,7 +26898,7 @@
         <v>679</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>1042</v>
+        <v>1040</v>
       </c>
       <c r="C36" s="27"/>
     </row>
@@ -26872,7 +26907,7 @@
         <v>87</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
       <c r="C37" s="22"/>
     </row>
@@ -26881,7 +26916,7 @@
         <v>117</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
       <c r="C38" s="27"/>
     </row>
@@ -26890,7 +26925,7 @@
         <v>123</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
       <c r="C39" s="22"/>
     </row>
@@ -26899,7 +26934,7 @@
         <v>135</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
       <c r="C40" s="22"/>
     </row>
@@ -26908,52 +26943,52 @@
         <v>146</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>1047</v>
+        <v>1045</v>
       </c>
       <c r="C41" s="22"/>
     </row>
     <row r="42" spans="1:3" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="26" t="s">
-        <v>1048</v>
+        <v>1046</v>
       </c>
       <c r="B42" s="26" t="s">
-        <v>1049</v>
+        <v>1047</v>
       </c>
       <c r="C42" s="27"/>
     </row>
     <row r="43" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="21" t="s">
-        <v>1050</v>
+        <v>1048</v>
       </c>
       <c r="B43" s="21" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
       <c r="C43" s="22"/>
     </row>
     <row r="44" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="21" t="s">
-        <v>1052</v>
+        <v>1050</v>
       </c>
       <c r="B44" s="21" t="s">
-        <v>1053</v>
+        <v>1051</v>
       </c>
       <c r="C44" s="22"/>
     </row>
     <row r="45" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="21" t="s">
-        <v>1054</v>
+        <v>1052</v>
       </c>
       <c r="B45" s="21" t="s">
-        <v>1055</v>
+        <v>1053</v>
       </c>
       <c r="C45" s="22"/>
     </row>
     <row r="46" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="21" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
       <c r="B46" s="21" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
       <c r="C46" s="22"/>
     </row>
@@ -26962,16 +26997,16 @@
         <v>225</v>
       </c>
       <c r="B47" s="26" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="C47" s="27"/>
     </row>
     <row r="48" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="21" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="B48" s="21" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
       <c r="C48" s="22"/>
     </row>
@@ -26980,61 +27015,61 @@
         <v>680</v>
       </c>
       <c r="B49" s="21" t="s">
-        <v>1061</v>
+        <v>1059</v>
       </c>
       <c r="C49" s="22"/>
     </row>
     <row r="50" spans="1:3" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="26" t="s">
-        <v>1062</v>
+        <v>1060</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>1063</v>
+        <v>1061</v>
       </c>
       <c r="C50" s="27"/>
     </row>
     <row r="51" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="26" t="s">
-        <v>1064</v>
+        <v>1062</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="C51" s="27"/>
     </row>
     <row r="52" spans="1:3" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="21" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
       <c r="B52" s="21" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="C52" s="22"/>
     </row>
     <row r="53" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="26" t="s">
-        <v>1068</v>
+        <v>1066</v>
       </c>
       <c r="B53" s="26" t="s">
-        <v>1069</v>
+        <v>1067</v>
       </c>
       <c r="C53" s="27"/>
     </row>
     <row r="54" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="21" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="B54" s="21" t="s">
-        <v>1071</v>
+        <v>1069</v>
       </c>
       <c r="C54" s="22"/>
     </row>
     <row r="55" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="26" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
       <c r="B55" s="26" t="s">
-        <v>1073</v>
+        <v>1071</v>
       </c>
       <c r="C55" s="27"/>
     </row>
@@ -27043,25 +27078,25 @@
         <v>217</v>
       </c>
       <c r="B56" s="26" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
       <c r="C56" s="27"/>
     </row>
     <row r="57" spans="1:3" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="26" t="s">
-        <v>1075</v>
+        <v>1073</v>
       </c>
       <c r="B57" s="26" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="C57" s="27"/>
     </row>
     <row r="58" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="26" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="B58" s="26" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
       <c r="C58" s="27"/>
     </row>
@@ -27070,34 +27105,34 @@
         <v>162</v>
       </c>
       <c r="B59" s="49" t="s">
-        <v>1095</v>
+        <v>1093</v>
       </c>
       <c r="C59" s="50"/>
     </row>
     <row r="60" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" s="49" t="s">
-        <v>1198</v>
+        <v>1196</v>
       </c>
       <c r="B60" s="49" t="s">
-        <v>1199</v>
+        <v>1197</v>
       </c>
       <c r="C60" s="50"/>
     </row>
     <row r="61" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="49" t="s">
-        <v>1256</v>
+        <v>1254</v>
       </c>
       <c r="B61" s="49" t="s">
-        <v>1259</v>
+        <v>1257</v>
       </c>
       <c r="C61" s="50"/>
     </row>
     <row r="62" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="49" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="B62" s="49" t="s">
-        <v>1260</v>
+        <v>1258</v>
       </c>
       <c r="C62" s="50"/>
     </row>
@@ -27121,18 +27156,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="B2" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -27140,7 +27175,7 @@
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -27148,7 +27183,7 @@
         <v>242</v>
       </c>
       <c r="B4" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -27156,7 +27191,7 @@
         <v>89</v>
       </c>
       <c r="B5" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
     </row>
   </sheetData>
@@ -27178,18 +27213,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="B2" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
     </row>
   </sheetData>
@@ -27217,7 +27252,7 @@
         <v>4</v>
       </c>
       <c r="B1" s="82" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -27225,7 +27260,7 @@
         <v>159</v>
       </c>
       <c r="B2" s="36" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -27233,31 +27268,31 @@
         <v>152</v>
       </c>
       <c r="B3" s="35" t="s">
-        <v>1085</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="68" t="s">
-        <v>1086</v>
+        <v>1084</v>
       </c>
       <c r="B4" s="36" t="s">
-        <v>1087</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="68" t="s">
-        <v>1088</v>
+        <v>1086</v>
       </c>
       <c r="B5" s="36" t="s">
-        <v>1089</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="83" t="s">
-        <v>1090</v>
+        <v>1088</v>
       </c>
       <c r="B6" s="83" t="s">
-        <v>1090</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -27270,10 +27305,10 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="68" t="s">
-        <v>1091</v>
+        <v>1089</v>
       </c>
       <c r="B8" s="68" t="s">
-        <v>1091</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -27318,26 +27353,26 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="68" t="s">
-        <v>1092</v>
+        <v>1090</v>
       </c>
       <c r="B14" s="68" t="s">
-        <v>1092</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="36" t="s">
-        <v>1093</v>
+        <v>1091</v>
       </c>
       <c r="B15" s="36" t="s">
-        <v>1093</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="68" t="s">
-        <v>1094</v>
+        <v>1092</v>
       </c>
       <c r="B16" s="68" t="s">
-        <v>1094</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
CD-182: Updated regex for 'orcid_id', 'library_prep_kit_version' and 'reference_genome' fields in Single-cell schema
- Updated regex for 'orcid_id' field to accept IDs ending with X as a checksum character
- Allow decimal values for the 'library_prep_kit_version' field
- Allow multiple URLs to be entered for 'reference_genome' field as a pipe symbol (|) separated entry
</commit_message>
<xml_diff>
--- a/single_cell/singlecell_schema_main_v0.4.xlsx
+++ b/single_cell/singlecell_schema_main_v0.4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/providen/Documents/EI/Projects/COPO-schemas/single_cell/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82992FDF-4828-5E4A-9195-C924823E24B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFBAD219-B085-E441-B2BB-170709C5D663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-2660" windowWidth="38400" windowHeight="21600" activeTab="1" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3128" uniqueCount="1272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3128" uniqueCount="1276">
   <si>
     <t>component_name</t>
   </si>
@@ -4029,6 +4029,18 @@
   </si>
   <si>
     <t>NOMe-Seq</t>
+  </si>
+  <si>
+    <t>^\d{4}-\d{4}-\d{4}-\d{3}[\dX]$</t>
+  </si>
+  <si>
+    <t>^((https?|ftp):\/\/[^\s|]+)(\|((https?|ftp):\/\/[^\s|]+))*$</t>
+  </si>
+  <si>
+    <t>Expected a URL starting with 'http', 'https' or 'ftp'. For multiple URLs, separate them using the pipe symbol (|) with no spaces. e.g. https://reference-genome-example.com|https://example.org</t>
+  </si>
+  <si>
+    <t>Expected positive whole numbers or decimal numbers.</t>
   </si>
 </sst>
 </file>
@@ -5011,10 +5023,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -6249,7 +6261,7 @@
         <v>110</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>111</v>
+        <v>1272</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>1223</v>
@@ -8543,10 +8555,10 @@
         <v>290</v>
       </c>
       <c r="K68" s="3" t="s">
-        <v>241</v>
+        <v>676</v>
       </c>
       <c r="L68" s="3" t="s">
-        <v>1226</v>
+        <v>1275</v>
       </c>
       <c r="M68" s="3" t="s">
         <v>24</v>
@@ -13398,7 +13410,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="176" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" s="8" t="s">
         <v>1103</v>
       </c>
@@ -13467,7 +13479,7 @@
       <c r="I177" s="3" t="s">
         <v>1123</v>
       </c>
-      <c r="J177" s="97" t="s">
+      <c r="J177" s="98" t="s">
         <v>1165</v>
       </c>
       <c r="M177" s="3" t="s">
@@ -13512,10 +13524,10 @@
         <v>1235</v>
       </c>
       <c r="K178" s="3" t="s">
-        <v>201</v>
+        <v>1273</v>
       </c>
       <c r="L178" s="3" t="s">
-        <v>1228</v>
+        <v>1274</v>
       </c>
       <c r="M178" s="3" t="s">
         <v>24</v>
@@ -13802,7 +13814,7 @@
       <c r="J185" s="95">
         <v>2.5</v>
       </c>
-      <c r="K185" s="98" t="s">
+      <c r="K185" s="97" t="s">
         <v>1252</v>
       </c>
       <c r="L185" t="s">
@@ -14626,6 +14638,7 @@
     <hyperlink ref="J178" r:id="rId59" xr:uid="{36FAB4CA-D2E7-2648-850A-DCF88860F33D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <legacyDrawing r:id="rId60"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
CD-187: Added missing regex to 'regex_to_formula' worksheet
- The regex for orcid_id and reference_genome were added to the worksheet.

- Added updated versions of json and yaml versions of the xlsx main schema
</commit_message>
<xml_diff>
--- a/single_cell/singlecell_schema_main_v0.4.xlsx
+++ b/single_cell/singlecell_schema_main_v0.4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/providen/Documents/EI/Projects/COPO-schemas/single_cell/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFBAD219-B085-E441-B2BB-170709C5D663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE3E9841-8636-BD49-912D-441E57B94B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1400" yWindow="4860" windowWidth="30240" windowHeight="17780" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
+    <workbookView xWindow="37020" yWindow="-140" windowWidth="27740" windowHeight="16420" activeTab="5" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3128" uniqueCount="1276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3132" uniqueCount="1278">
   <si>
     <t>component_name</t>
   </si>
@@ -4041,6 +4041,12 @@
   </si>
   <si>
     <t>Expected positive whole numbers or decimal numbers.</t>
+  </si>
+  <si>
+    <t>AND(LEN(A1)=19,MID(A1,5,1)="-",MID(A1,10,1)="-",MID(A1,15,1)="-",ISNUMBER(--LEFT(A1,4)),ISNUMBER(--MID(A1,6,4)),ISNUMBER(--MID(A1,11,4)),ISNUMBER(--MID(A1,16,3)),OR(ISNUMBER(--RIGHT(A1,1)),RIGHT(A1,1)="X"))</t>
+  </si>
+  <si>
+    <t>OR(LEFT(A1,7)="http://",LEFT(A1,8)="https://",LEFT(A1,6)="ftp://")</t>
   </si>
 </sst>
 </file>
@@ -4761,7 +4767,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5024,9 +5030,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -13479,7 +13482,7 @@
       <c r="I177" s="3" t="s">
         <v>1123</v>
       </c>
-      <c r="J177" s="98" t="s">
+      <c r="J177" s="68" t="s">
         <v>1165</v>
       </c>
       <c r="M177" s="3" t="s">
@@ -26527,7 +26530,7 @@
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="41.5" style="19" customWidth="1"/>
@@ -27140,7 +27143,7 @@
       </c>
       <c r="C61" s="50"/>
     </row>
-    <row r="62" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:3" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="49" t="s">
         <v>1208</v>
       </c>
@@ -27148,6 +27151,24 @@
         <v>1258</v>
       </c>
       <c r="C62" s="50"/>
+    </row>
+    <row r="63" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="49" t="s">
+        <v>1273</v>
+      </c>
+      <c r="B63" s="49" t="s">
+        <v>1277</v>
+      </c>
+      <c r="C63" s="50"/>
+    </row>
+    <row r="64" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="49" t="s">
+        <v>1272</v>
+      </c>
+      <c r="B64" s="49" t="s">
+        <v>1276</v>
+      </c>
+      <c r="C64" s="50"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:C53" xr:uid="{D95B3E19-31EE-401E-8E14-DBEF7BC74F95}"/>

</xml_diff>

<commit_message>
CD-213: Ensure that `cell_number` field is included only in ToL Single-cell manifests and `cell_count` in non-ToL manifests
- `cell_number` is a similar field to `cell_count`. However, the `cell_number` field  should only be in ToL single-cell manifests and `cell_count` should be included in manifests that are not ToL
- This commit realises that logic.
</commit_message>
<xml_diff>
--- a/single_cell/singlecell_schema_main_v0.4.xlsx
+++ b/single_cell/singlecell_schema_main_v0.4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/providen/Documents/EI/Projects/COPO-schemas/single_cell/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD285F8-18DE-8342-A1C5-ADEBD729A9AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C676717-8F39-4245-86B4-5287FEA13904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-2660" windowWidth="38400" windowHeight="21600" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
+    <workbookView xWindow="32460" yWindow="-1460" windowWidth="28920" windowHeight="15720" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3096" uniqueCount="1266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3094" uniqueCount="1266">
   <si>
     <t>component_name</t>
   </si>
@@ -7811,9 +7811,7 @@
       <c r="Q52" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="R52" s="56" t="s">
-        <v>27</v>
-      </c>
+      <c r="R52" s="56"/>
       <c r="S52" s="85" t="s">
         <v>27</v>
       </c>
@@ -7857,9 +7855,7 @@
       <c r="R53" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="S53" s="85" t="s">
-        <v>27</v>
-      </c>
+      <c r="S53" s="85"/>
     </row>
     <row r="54" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" s="8" t="s">

</xml_diff>